<commit_message>
docs: publish Vera usage declarations and update assessment
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R759e930075f74ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7f4fc1c70266440d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -49,6 +49,12 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF315D88"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0070C0"/>
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
@@ -99,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -166,6 +172,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -383,7 +398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
@@ -447,12 +462,12 @@
       </x:c>
       <x:c r="F5" s="8" t="inlineStr">
         <x:is>
-          <x:t>Finalità</x:t>
+          <x:t xml:space="preserve">Finalità</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" s="8" t="inlineStr">
         <x:is>
-          <x:t>Riferimento normativo</x:t>
+          <x:t xml:space="preserve">Riferimento normativo</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -475,12 +490,12 @@
       </x:c>
       <x:c r="F6" s="12" t="inlineStr">
         <x:is>
-          <x:t>Ridurre i dati trasmessi a terzi</x:t>
+          <x:t xml:space="preserve">Ridurre i dati trasmessi a terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="12" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. c); 25, par. 2 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. c); 25, par. 2 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -503,12 +518,12 @@
       </x:c>
       <x:c r="F7" s="13" t="inlineStr">
         <x:is>
-          <x:t>Inviare solo i dati necessari alla finalità</x:t>
+          <x:t xml:space="preserve">Inviare solo i dati necessari alla finalità</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. c); 25 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. c); 25 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -531,12 +546,12 @@
       </x:c>
       <x:c r="F8" s="14" t="inlineStr">
         <x:is>
-          <x:t>Accountability dello studio; base per il registro dei trattamenti</x:t>
+          <x:t xml:space="preserve">Accountability dello studio; base per il registro dei trattamenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 2; 30 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 2; 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -559,12 +574,12 @@
       </x:c>
       <x:c r="F9" s="13" t="inlineStr">
         <x:is>
-          <x:t>Ridurre l'identificabilità dei dati inviati</x:t>
+          <x:t xml:space="preserve">Ridurre l'identificabilità dei dati inviati</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 n. 5 GDPR; considerando 26</x:t>
+          <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -587,12 +602,12 @@
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
-          <x:t>Evitare l'ingresso degli sviluppatori nel trattamento</x:t>
+          <x:t xml:space="preserve">Evitare l'ingresso degli sviluppatori nel trattamento</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 4 n. 7-8, 25, 28 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 4 n. 7-8, 25, 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -615,12 +630,12 @@
       </x:c>
       <x:c r="F11" s="13" t="inlineStr">
         <x:is>
-          <x:t>Garantire la base contrattuale con il provider</x:t>
+          <x:t xml:space="preserve">Garantire la base contrattuale con il provider</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -643,12 +658,12 @@
       </x:c>
       <x:c r="F12" s="14" t="inlineStr">
         <x:is>
-          <x:t>Informare lo studio sulle condizioni di ciascuna piattaforma</x:t>
+          <x:t xml:space="preserve">Informare lo studio sulle condizioni di ciascuna piattaforma</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 28, 44 ss. GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -671,12 +686,12 @@
       </x:c>
       <x:c r="F13" s="13" t="inlineStr">
         <x:is>
-          <x:t>Ridurre il rischio di invio di dati ad alto impatto</x:t>
+          <x:t xml:space="preserve">Ridurre il rischio di invio di dati ad alto impatto</x:t>
         </x:is>
       </x:c>
       <x:c r="G13" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 9, 10 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 9, 10 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -699,12 +714,12 @@
       </x:c>
       <x:c r="F14" s="14" t="inlineStr">
         <x:is>
-          <x:t>Sicurezza, tracciabilità, limitazione della conservazione</x:t>
+          <x:t xml:space="preserve">Sicurezza, tracciabilità, limitazione della conservazione</x:t>
         </x:is>
       </x:c>
       <x:c r="G14" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. e); 32 GDPR; Provv. Garante 27/11/2008</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. e); 32 GDPR; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -726,12 +741,12 @@
       </x:c>
       <x:c r="F15" s="13" t="inlineStr">
         <x:is>
-          <x:t>Sicurezza del trattamento</x:t>
+          <x:t xml:space="preserve">Sicurezza del trattamento</x:t>
         </x:is>
       </x:c>
       <x:c r="G15" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 32 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 32 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -754,12 +769,12 @@
       </x:c>
       <x:c r="F16" s="14" t="inlineStr">
         <x:is>
-          <x:t>Prevalenza dell'attività intellettuale umana e responsabilità del professionista</x:t>
+          <x:t xml:space="preserve">Prevalenza dell'attività intellettuale umana e responsabilità del professionista</x:t>
         </x:is>
       </x:c>
       <x:c r="G16" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 13, co. 1, L. 132/2025; art. 21, co. 8-10, Codice deontologico CNDCEC</x:t>
+          <x:t xml:space="preserve">Art. 13, co. 1, L. 132/2025; art. 21, co. 8-10, Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -782,12 +797,12 @@
       </x:c>
       <x:c r="F17" s="13" t="inlineStr">
         <x:is>
-          <x:t>Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
+          <x:t xml:space="preserve">Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
         </x:is>
       </x:c>
       <x:c r="G17" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
+          <x:t xml:space="preserve">Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -810,12 +825,12 @@
       </x:c>
       <x:c r="F18" s="14" t="inlineStr">
         <x:is>
-          <x:t>Trasparenza e tracciabilità dei rilasci</x:t>
+          <x:t xml:space="preserve">Trasparenza e tracciabilità dei rilasci</x:t>
         </x:is>
       </x:c>
       <x:c r="G18" s="14" t="inlineStr">
         <x:is>
-          <x:t>—</x:t>
+          <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -838,12 +853,12 @@
       </x:c>
       <x:c r="F19" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supportare l'adempimento dell'art. 30</x:t>
+          <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
       <x:c r="G19" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 30 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -866,12 +881,12 @@
       </x:c>
       <x:c r="F20" s="14" t="inlineStr">
         <x:is>
-          <x:t>Orientare la valutazione sulla necessità della DPIA</x:t>
+          <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
       <x:c r="G20" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 35 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -894,12 +909,12 @@
       </x:c>
       <x:c r="F21" s="13" t="inlineStr">
         <x:is>
-          <x:t>Informativa privacy e informativa IA</x:t>
+          <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
       <x:c r="G21" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
+          <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -921,12 +936,12 @@
       </x:c>
       <x:c r="F22" s="14" t="inlineStr">
         <x:is>
-          <x:t>Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -948,12 +963,12 @@
       </x:c>
       <x:c r="F23" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="13" t="inlineStr">
         <x:is>
-          <x:t>Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -976,12 +991,12 @@
       </x:c>
       <x:c r="F24" s="14" t="inlineStr">
         <x:is>
-          <x:t>Governo dell'uso dell'IA nello studio</x:t>
+          <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="14" t="inlineStr">
         <x:is>
-          <x:t>AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
+          <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1004,12 +1019,12 @@
       </x:c>
       <x:c r="F25" s="13" t="inlineStr">
         <x:is>
-          <x:t>Dimostrare le attività di alfabetizzazione</x:t>
+          <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 AI Act (testo modificato)</x:t>
+          <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1031,12 +1046,12 @@
       </x:c>
       <x:c r="F26" s="14" t="inlineStr">
         <x:is>
-          <x:t>Preparare la risposta a incidenti</x:t>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 33-34 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1059,12 +1074,12 @@
       </x:c>
       <x:c r="F27" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supporto alla trasparenza verso clienti e terzi</x:t>
+          <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G27" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 13, co. 2, L. 132/2025</x:t>
+          <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1086,12 +1101,12 @@
       </x:c>
       <x:c r="F28" s="14" t="inlineStr">
         <x:is>
-          <x:t>Istruzioni e designazioni all'interno dello studio</x:t>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G28" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1099,27 +1114,27 @@
       <x:c r="A29" s="13" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B29" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C29" s="13" t="str">
-        <x:v>Il registro tecnico esplicita che non costituisce prova o certificazione della conformità GDPR. Descrive i flussi e i controlli del prodotto.</x:v>
+        <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
       <x:c r="D29" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E29" s="21" t="str">
-        <x:v>Confini del registro tecnico
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/privacy-surface-review/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.1
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
       <x:c r="F29" s="13" t="inlineStr">
         <x:is>
-          <x:t>Evitare affidamento improprio</x:t>
+          <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
       <x:c r="G29" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 4 n. 7, 24 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1127,27 +1142,27 @@
       <x:c r="A30" s="14" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B30" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>I profili riferiscono il trattamento all’account e al rapporto con la piattaforma scelti dallo studio. Il plugin non stipula né verifica il contratto.</x:v>
+        <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E30" s="22" t="str">
-        <x:v>Assetto dell’account scelto dallo studio
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.2
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
       <x:c r="F30" s="14" t="inlineStr">
         <x:is>
-          <x:t>Chiarire la responsabilità dello studio</x:t>
+          <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G30" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1155,27 +1170,27 @@
       <x:c r="A31" s="13" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C31" s="13" t="str">
-        <x:v>La guida del connettore descrive placeholder, possibili dati residui e limiti del filtraggio. Non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
+        <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
       <x:c r="D31" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E31" s="21" t="str">
-        <x:v>Limiti del filtro e assenza di garanzia di anonimato
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/connectors/privacy-filter/README.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.3
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
       <x:c r="F31" s="13" t="inlineStr">
         <x:is>
-          <x:t>Evitare l'affidamento sull'"anonimo"</x:t>
+          <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
       <x:c r="G31" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 n. 5 GDPR; considerando 26</x:t>
+          <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1183,27 +1198,27 @@
       <x:c r="A32" s="14" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B32" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>Il plugin non verifica il piano né applica una regola di esclusione degli account consumer. I profili rinviano alle condizioni dell’account scelto.</x:v>
+        <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E32" s="22" t="str">
-        <x:v>Contratti e piano: assunzioni esterne
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.4
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
       <x:c r="F32" s="14" t="inlineStr">
         <x:is>
-          <x:t>Delimitare il perimetro d'uso</x:t>
+          <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
       <x:c r="G32" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1211,27 +1226,27 @@
       <x:c r="A33" s="13" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C33" s="13" t="str">
-        <x:v>I profili esplicitano che piano, retention e controlli del provider dipendono dall’account scelto e non sono imposti da Vera.</x:v>
+        <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E33" s="21" t="str">
-        <x:v>Limiti rispetto alla piattaforma
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.5
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
       <x:c r="F33" s="13" t="inlineStr">
         <x:is>
-          <x:t>Chiarire i limiti rispetto ai terzi</x:t>
+          <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G33" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 28, 44 ss. GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1239,27 +1254,27 @@
       <x:c r="A34" s="14" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B34" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>Vera prepara anche bozze di pareri; i workflow richiedono fonti, revisione e giudizio professionale. L’approvazione non è effettuata dal software.</x:v>
+        <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E34" s="22" t="str">
-        <x:v>Bozze, validazione e provenienza del lavoro
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.6
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
       <x:c r="F34" s="14" t="inlineStr">
         <x:is>
-          <x:t>Prevalenza del giudizio umano</x:t>
+          <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
       <x:c r="G34" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
+          <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1267,27 +1282,27 @@
       <x:c r="A35" s="15" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B35" s="19" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B35" s="26" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>L’avviso sull’aggiornamento normativo va inserito nella documentazione d’uso insieme alle altre dichiarazioni.</x:v>
+        <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>Redigere e inserire nella documentazione d’uso di Vera l’avviso sull’aggiornamento normativo, con la data di verifica dei riferimenti e l’invito alla verifica sulle fonti ufficiali.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Ricerca su fonti attuali e validazione delle risposte
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.7
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
       <x:c r="F35" s="15" t="inlineStr">
         <x:is>
-          <x:t>Evitare obsolescenza non dichiarata</x:t>
+          <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
       <x:c r="G35" s="15" t="inlineStr">
         <x:is>
-          <x:t>—</x:t>
+          <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1299,7 +1314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rb0117e71120b4003"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd61e37ba7e584049"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: publish Vera usage declarations and update assessment (#766)
Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R759e930075f74ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7f4fc1c70266440d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -49,6 +49,12 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF315D88"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0070C0"/>
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
@@ -99,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -166,6 +172,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -383,7 +398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
@@ -447,12 +462,12 @@
       </x:c>
       <x:c r="F5" s="8" t="inlineStr">
         <x:is>
-          <x:t>Finalità</x:t>
+          <x:t xml:space="preserve">Finalità</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" s="8" t="inlineStr">
         <x:is>
-          <x:t>Riferimento normativo</x:t>
+          <x:t xml:space="preserve">Riferimento normativo</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -475,12 +490,12 @@
       </x:c>
       <x:c r="F6" s="12" t="inlineStr">
         <x:is>
-          <x:t>Ridurre i dati trasmessi a terzi</x:t>
+          <x:t xml:space="preserve">Ridurre i dati trasmessi a terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="12" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. c); 25, par. 2 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. c); 25, par. 2 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -503,12 +518,12 @@
       </x:c>
       <x:c r="F7" s="13" t="inlineStr">
         <x:is>
-          <x:t>Inviare solo i dati necessari alla finalità</x:t>
+          <x:t xml:space="preserve">Inviare solo i dati necessari alla finalità</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. c); 25 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. c); 25 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -531,12 +546,12 @@
       </x:c>
       <x:c r="F8" s="14" t="inlineStr">
         <x:is>
-          <x:t>Accountability dello studio; base per il registro dei trattamenti</x:t>
+          <x:t xml:space="preserve">Accountability dello studio; base per il registro dei trattamenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 2; 30 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 2; 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -559,12 +574,12 @@
       </x:c>
       <x:c r="F9" s="13" t="inlineStr">
         <x:is>
-          <x:t>Ridurre l'identificabilità dei dati inviati</x:t>
+          <x:t xml:space="preserve">Ridurre l'identificabilità dei dati inviati</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 n. 5 GDPR; considerando 26</x:t>
+          <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -587,12 +602,12 @@
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
-          <x:t>Evitare l'ingresso degli sviluppatori nel trattamento</x:t>
+          <x:t xml:space="preserve">Evitare l'ingresso degli sviluppatori nel trattamento</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 4 n. 7-8, 25, 28 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 4 n. 7-8, 25, 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -615,12 +630,12 @@
       </x:c>
       <x:c r="F11" s="13" t="inlineStr">
         <x:is>
-          <x:t>Garantire la base contrattuale con il provider</x:t>
+          <x:t xml:space="preserve">Garantire la base contrattuale con il provider</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -643,12 +658,12 @@
       </x:c>
       <x:c r="F12" s="14" t="inlineStr">
         <x:is>
-          <x:t>Informare lo studio sulle condizioni di ciascuna piattaforma</x:t>
+          <x:t xml:space="preserve">Informare lo studio sulle condizioni di ciascuna piattaforma</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 28, 44 ss. GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -671,12 +686,12 @@
       </x:c>
       <x:c r="F13" s="13" t="inlineStr">
         <x:is>
-          <x:t>Ridurre il rischio di invio di dati ad alto impatto</x:t>
+          <x:t xml:space="preserve">Ridurre il rischio di invio di dati ad alto impatto</x:t>
         </x:is>
       </x:c>
       <x:c r="G13" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 9, 10 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 9, 10 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -699,12 +714,12 @@
       </x:c>
       <x:c r="F14" s="14" t="inlineStr">
         <x:is>
-          <x:t>Sicurezza, tracciabilità, limitazione della conservazione</x:t>
+          <x:t xml:space="preserve">Sicurezza, tracciabilità, limitazione della conservazione</x:t>
         </x:is>
       </x:c>
       <x:c r="G14" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 5, par. 1, lett. e); 32 GDPR; Provv. Garante 27/11/2008</x:t>
+          <x:t xml:space="preserve">Artt. 5, par. 1, lett. e); 32 GDPR; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -726,12 +741,12 @@
       </x:c>
       <x:c r="F15" s="13" t="inlineStr">
         <x:is>
-          <x:t>Sicurezza del trattamento</x:t>
+          <x:t xml:space="preserve">Sicurezza del trattamento</x:t>
         </x:is>
       </x:c>
       <x:c r="G15" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 32 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 32 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -754,12 +769,12 @@
       </x:c>
       <x:c r="F16" s="14" t="inlineStr">
         <x:is>
-          <x:t>Prevalenza dell'attività intellettuale umana e responsabilità del professionista</x:t>
+          <x:t xml:space="preserve">Prevalenza dell'attività intellettuale umana e responsabilità del professionista</x:t>
         </x:is>
       </x:c>
       <x:c r="G16" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 13, co. 1, L. 132/2025; art. 21, co. 8-10, Codice deontologico CNDCEC</x:t>
+          <x:t xml:space="preserve">Art. 13, co. 1, L. 132/2025; art. 21, co. 8-10, Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -782,12 +797,12 @@
       </x:c>
       <x:c r="F17" s="13" t="inlineStr">
         <x:is>
-          <x:t>Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
+          <x:t xml:space="preserve">Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
         </x:is>
       </x:c>
       <x:c r="G17" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
+          <x:t xml:space="preserve">Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -810,12 +825,12 @@
       </x:c>
       <x:c r="F18" s="14" t="inlineStr">
         <x:is>
-          <x:t>Trasparenza e tracciabilità dei rilasci</x:t>
+          <x:t xml:space="preserve">Trasparenza e tracciabilità dei rilasci</x:t>
         </x:is>
       </x:c>
       <x:c r="G18" s="14" t="inlineStr">
         <x:is>
-          <x:t>—</x:t>
+          <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -838,12 +853,12 @@
       </x:c>
       <x:c r="F19" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supportare l'adempimento dell'art. 30</x:t>
+          <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
       <x:c r="G19" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 30 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -866,12 +881,12 @@
       </x:c>
       <x:c r="F20" s="14" t="inlineStr">
         <x:is>
-          <x:t>Orientare la valutazione sulla necessità della DPIA</x:t>
+          <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
       <x:c r="G20" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 35 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -894,12 +909,12 @@
       </x:c>
       <x:c r="F21" s="13" t="inlineStr">
         <x:is>
-          <x:t>Informativa privacy e informativa IA</x:t>
+          <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
       <x:c r="G21" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
+          <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -921,12 +936,12 @@
       </x:c>
       <x:c r="F22" s="14" t="inlineStr">
         <x:is>
-          <x:t>Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -948,12 +963,12 @@
       </x:c>
       <x:c r="F23" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="13" t="inlineStr">
         <x:is>
-          <x:t>Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -976,12 +991,12 @@
       </x:c>
       <x:c r="F24" s="14" t="inlineStr">
         <x:is>
-          <x:t>Governo dell'uso dell'IA nello studio</x:t>
+          <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="14" t="inlineStr">
         <x:is>
-          <x:t>AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
+          <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1004,12 +1019,12 @@
       </x:c>
       <x:c r="F25" s="13" t="inlineStr">
         <x:is>
-          <x:t>Dimostrare le attività di alfabetizzazione</x:t>
+          <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 AI Act (testo modificato)</x:t>
+          <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1031,12 +1046,12 @@
       </x:c>
       <x:c r="F26" s="14" t="inlineStr">
         <x:is>
-          <x:t>Preparare la risposta a incidenti</x:t>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="14" t="inlineStr">
         <x:is>
-          <x:t>Artt. 33-34 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1059,12 +1074,12 @@
       </x:c>
       <x:c r="F27" s="13" t="inlineStr">
         <x:is>
-          <x:t>Supporto alla trasparenza verso clienti e terzi</x:t>
+          <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G27" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 13, co. 2, L. 132/2025</x:t>
+          <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1086,12 +1101,12 @@
       </x:c>
       <x:c r="F28" s="14" t="inlineStr">
         <x:is>
-          <x:t>Istruzioni e designazioni all'interno dello studio</x:t>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G28" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1099,27 +1114,27 @@
       <x:c r="A29" s="13" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B29" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C29" s="13" t="str">
-        <x:v>Il registro tecnico esplicita che non costituisce prova o certificazione della conformità GDPR. Descrive i flussi e i controlli del prodotto.</x:v>
+        <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
       <x:c r="D29" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E29" s="21" t="str">
-        <x:v>Confini del registro tecnico
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/privacy-surface-review/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.1
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
       <x:c r="F29" s="13" t="inlineStr">
         <x:is>
-          <x:t>Evitare affidamento improprio</x:t>
+          <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
       <x:c r="G29" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 4 n. 7, 24 GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1127,27 +1142,27 @@
       <x:c r="A30" s="14" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B30" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B30" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
-        <x:v>I profili riferiscono il trattamento all’account e al rapporto con la piattaforma scelti dallo studio. Il plugin non stipula né verifica il contratto.</x:v>
+        <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E30" s="22" t="str">
-        <x:v>Assetto dell’account scelto dallo studio
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.2
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
       <x:c r="F30" s="14" t="inlineStr">
         <x:is>
-          <x:t>Chiarire la responsabilità dello studio</x:t>
+          <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
       <x:c r="G30" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1155,27 +1170,27 @@
       <x:c r="A31" s="13" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C31" s="13" t="str">
-        <x:v>La guida del connettore descrive placeholder, possibili dati residui e limiti del filtraggio. Non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
+        <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
       <x:c r="D31" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E31" s="21" t="str">
-        <x:v>Limiti del filtro e assenza di garanzia di anonimato
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/connectors/privacy-filter/README.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.3
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
       <x:c r="F31" s="13" t="inlineStr">
         <x:is>
-          <x:t>Evitare l'affidamento sull'"anonimo"</x:t>
+          <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
       <x:c r="G31" s="13" t="inlineStr">
         <x:is>
-          <x:t>Art. 4 n. 5 GDPR; considerando 26</x:t>
+          <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1183,27 +1198,27 @@
       <x:c r="A32" s="14" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B32" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C32" s="14" t="str">
-        <x:v>Il plugin non verifica il piano né applica una regola di esclusione degli account consumer. I profili rinviano alle condizioni dell’account scelto.</x:v>
+        <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
       <x:c r="D32" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E32" s="22" t="str">
-        <x:v>Contratti e piano: assunzioni esterne
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.4
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
       <x:c r="F32" s="14" t="inlineStr">
         <x:is>
-          <x:t>Delimitare il perimetro d'uso</x:t>
+          <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
       <x:c r="G32" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 28 GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1211,27 +1226,27 @@
       <x:c r="A33" s="13" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C33" s="13" t="str">
-        <x:v>I profili esplicitano che piano, retention e controlli del provider dipendono dall’account scelto e non sono imposti da Vera.</x:v>
+        <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E33" s="21" t="str">
-        <x:v>Limiti rispetto alla piattaforma
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/privacy/runtime-profiles.json</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.5
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
       <x:c r="F33" s="13" t="inlineStr">
         <x:is>
-          <x:t>Chiarire i limiti rispetto ai terzi</x:t>
+          <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
       <x:c r="G33" s="13" t="inlineStr">
         <x:is>
-          <x:t>Artt. 28, 44 ss. GDPR</x:t>
+          <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1239,27 +1254,27 @@
       <x:c r="A34" s="14" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B34" s="18" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C34" s="14" t="str">
-        <x:v>Vera prepara anche bozze di pareri; i workflow richiedono fonti, revisione e giudizio professionale. L’approvazione non è effettuata dal software.</x:v>
+        <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
       <x:c r="D34" s="14" t="str">
-        <x:v>Redigere e inserire questa dichiarazione nella documentazione d’uso di Vera, in una sezione dedicata alle condizioni e ai limiti d’uso.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E34" s="22" t="str">
-        <x:v>Bozze, validazione e provenienza del lavoro
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.6
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
       <x:c r="F34" s="14" t="inlineStr">
         <x:is>
-          <x:t>Prevalenza del giudizio umano</x:t>
+          <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
       <x:c r="G34" s="14" t="inlineStr">
         <x:is>
-          <x:t>Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
+          <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1267,27 +1282,27 @@
       <x:c r="A35" s="15" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B35" s="19" t="str">
-        <x:v>Da implementare</x:v>
+      <x:c r="B35" s="26" t="str">
+        <x:v>Presente</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>L’avviso sull’aggiornamento normativo va inserito nella documentazione d’uso insieme alle altre dichiarazioni.</x:v>
+        <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>Redigere e inserire nella documentazione d’uso di Vera l’avviso sull’aggiornamento normativo, con la data di verifica dei riferimenti e l’invito alla verifica sulle fonti ufficiali.</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="E35" s="23" t="str">
-        <x:v>Ricerca su fonti attuali e validazione delle risposte
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
+        <x:v>Condizioni e limiti d’uso di Vera — N3.7
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
       <x:c r="F35" s="15" t="inlineStr">
         <x:is>
-          <x:t>Evitare obsolescenza non dichiarata</x:t>
+          <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
       <x:c r="G35" s="15" t="inlineStr">
         <x:is>
-          <x:t>—</x:t>
+          <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1299,7 +1314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart ns1:id="Rb0117e71120b4003"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd61e37ba7e584049"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: clarify Vera open source and platform choice
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7f4fc1c70266440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rb7d4a3e875584685"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -619,7 +619,7 @@
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>Il piano e il contratto della piattaforma sono condizioni d’uso esterne a Vera. Il plugin non le verifica né le impone.</x:v>
+        <x:v>Vera non è legata a un’unica piattaforma: funziona con Codex, Cowork e Antigravity e può essere utilizzata anche con modelli locali, con funzionalità che dipendono dall’ambiente scelto. Il piano e il contratto della piattaforma sono condizioni d’uso esterne a Vera. Il plugin non le verifica né le impone.</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
         <x:v>—</x:v>
@@ -814,7 +814,7 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Il manifest dichiara versione e licenza; il repository conserva la cronologia delle modifiche.</x:v>
+        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>—</x:v>
@@ -1314,7 +1314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd61e37ba7e584049"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf3644ce8614fb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: clarify Vera open source and platform choice (#772)
Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7f4fc1c70266440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rb7d4a3e875584685"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -619,7 +619,7 @@
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C11" s="13" t="str">
-        <x:v>Il piano e il contratto della piattaforma sono condizioni d’uso esterne a Vera. Il plugin non le verifica né le impone.</x:v>
+        <x:v>Vera non è legata a un’unica piattaforma: funziona con Codex, Cowork e Antigravity e può essere utilizzata anche con modelli locali, con funzionalità che dipendono dall’ambiente scelto. Il piano e il contratto della piattaforma sono condizioni d’uso esterne a Vera. Il plugin non le verifica né le impone.</x:v>
       </x:c>
       <x:c r="D11" s="13" t="str">
         <x:v>—</x:v>
@@ -814,7 +814,7 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Il manifest dichiara versione e licenza; il repository conserva la cronologia delle modifiche.</x:v>
+        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>—</x:v>
@@ -1314,7 +1314,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd61e37ba7e584049"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf3644ce8614fb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: align Vera compliance assessment with schema 0.2
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rb7d4a3e875584685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdc79cf7a785e4608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -181,6 +181,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -191,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G35"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G37"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Voce dello schema"/>
     <x:tableColumn id="2" name="Stato attuale"/>
@@ -428,9 +437,9 @@
       <x:c r="D2" s="3"/>
       <x:c r="E2" s="3"/>
     </x:row>
-    <x:row r="3" ht="26" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>I rapporti con le piattaforme sono trattati come condizioni d’uso. Il connettore di anonimizzazione è opzionale. Base tecnica: sorgente pubblico Vera 0.1.338, 03/10/2026.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026. Riscontro aggiornato al 04/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -778,32 +787,32 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17" ht="92" customHeight="1">
+    <x:row r="17" ht="175" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>G1.12 — Censimento delle skill rispetto all'All. III AI Act e agli artt. 5 e 50, con indicazione di quelle che profilano persone fisiche</x:v>
+        <x:v>G1.12 — Analisi funzione per funzione rispetto all'All. III AI Act e all'art. 6, par. 3, con indicazione di quelle che trattano persone fisiche e producono valutazioni, punteggi o classificazioni</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>Presente</x:v>
+        <x:v>Da implementare</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>Il catalogo descrive le funzioni e i relativi flussi. Nessuna di queste funzioni effettua profilazione di persone fisiche.</x:v>
+        <x:v>Il catalogo descrive le funzioni e i relativi flussi. New Client e la revisione antiriciclaggio trattano anche dati di persone fisiche e includono valutazioni di rischio con revisione professionale. Non è ancora pubblicata l’analisi funzione per funzione richiesta dallo schema 0.2.</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>Documentare, per ciascuna funzione, finalità, persone interessate, valutazioni prodotte e confronto con l’Allegato III e l’art. 6, par. 3. Si tratta di un’analisi da redigere, non di una nuova funzione del software.</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
-        <x:v>Catalogo delle funzioni e degli usi supportati
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/workflow-catalog.md</x:v>
-      </x:c>
-      <x:c r="F17" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G17" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
-        </x:is>
+        <x:v>Catalogo di Vera
+https://mparanza.com/static/shared/vera/index.html?lang=it#core
+Fascicolo cliente
+https://mparanza.com/static/shared/new-client/index.html?lang=it
+Revisione antiriciclaggio
+https://mparanza.com/static/shared/aml-review/index.html?lang=it</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>Presidiare l'esenzione open source e il rischio di alto rischio</x:v>
+      </x:c>
+      <x:c r="G17" s="13" t="str">
+        <x:v>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="92" customHeight="1">
@@ -834,126 +843,125 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19" ht="92" customHeight="1">
+    <x:row r="19" ht="150" customHeight="1">
       <x:c r="A19" s="13" t="str">
+        <x:v>G1.14 — Marcatura leggibile dalle macchine dei testi generati e rilevabilità come generati artificialmente</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>Non previsto</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>Non è prevista in Vera una funzione dedicata alla marcatura leggibile dalle macchine dei testi generati. L’eventuale marcatura applicata dalla piattaforma AI non è verificata in questo riscontro. La nota visibile sull’uso dell’IA proposta in D2.9 è una funzione distinta.</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E19" s="21" t="str">
+        <x:v>Nota visibile sull’uso dell’IA
+https://mparanza.com/static/shared/vera-compliance/index.html#d2-9
+Art. 50: testo della norma
+https://ai-act-service-desk.ec.europa.eu/en/ai-act/article-50</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="str">
+        <x:v>Rispettare l'obbligo dei fornitori di sistemi che generano testo sintetico</x:v>
+      </x:c>
+      <x:c r="G19" s="13" t="str">
+        <x:v>Art. 50, par. 2 AI Act; art. 111, par. 4 (Reg. UE 2026/1744)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="92" customHeight="1">
+      <x:c r="A20" s="14" t="str">
         <x:v>D2.1 — Bozza di registro dei trattamenti alimentata dai report di elaborazione</x:v>
       </x:c>
-      <x:c r="B19" s="17" t="str">
+      <x:c r="B20" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C19" s="13" t="str">
+      <x:c r="C20" s="14" t="str">
         <x:v>I report di Vera possono fornire informazioni sulle lavorazioni svolte e sui dati utilizzati.</x:v>
       </x:c>
-      <x:c r="D19" s="13" t="str">
+      <x:c r="D20" s="14" t="str">
         <x:v>Implementare la generazione di una bozza del registro dei trattamenti, integrando i report di Vera con le informazioni fornite dallo studio.</x:v>
       </x:c>
-      <x:c r="E19" s="21" t="str">
+      <x:c r="E20" s="22" t="str">
         <x:v>Report di esecuzione e dati già disponibili
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/model-data-report-contract.md</x:v>
       </x:c>
-      <x:c r="F19" s="13" t="inlineStr">
+      <x:c r="F20" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
-      <x:c r="G19" s="13" t="inlineStr">
+      <x:c r="G20" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="20" ht="92" customHeight="1">
-      <x:c r="A20" s="14" t="str">
+    <x:row r="21" ht="92" customHeight="1">
+      <x:c r="A21" s="13" t="str">
         <x:v>D2.2 — Scheda di screening preliminare per la DPIA</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str">
+      <x:c r="B21" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C21" s="13" t="str">
         <x:v>Vera dispone di percorsi di raccolta delle informazioni e analisi con fonti; la scheda dedicata di screening DPIA resta da implementare.</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="D21" s="13" t="str">
         <x:v>Implementare un percorso guidato che raccolga i fatti sul trattamento, li valuti rispetto ai criteri pertinenti e produca una scheda di screening DPIA motivata, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E20" s="22" t="str">
+      <x:c r="E21" s="21" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F20" s="14" t="inlineStr">
+      <x:c r="F21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G20" s="14" t="inlineStr">
+      <x:c r="G21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21" ht="92" customHeight="1">
-      <x:c r="A21" s="13" t="str">
+    <x:row r="22" ht="92" customHeight="1">
+      <x:c r="A22" s="14" t="str">
         <x:v>D2.3 — Bozza di informativa ai clienti con clausola sull'uso dell'IA</x:v>
       </x:c>
-      <x:c r="B21" s="17" t="str">
+      <x:c r="B22" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C22" s="14" t="str">
         <x:v>New Client raccoglie informazioni privacy/IA e prepara un piano documentale; non produce la bozza dell’informativa richiesta.</x:v>
       </x:c>
-      <x:c r="D21" s="13" t="str">
+      <x:c r="D22" s="14" t="str">
         <x:v>Implementare la generazione di una bozza di informativa ai clienti con clausola sull’uso dell’IA, sulla base delle informazioni dello studio e delle fonti pertinenti, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E21" s="21" t="str">
+      <x:c r="E22" s="22" t="str">
         <x:v>Applicabilità privacy/IA e piano documentale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/new-client/skills/new-client/SKILL.md</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="inlineStr">
+      <x:c r="F22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G21" s="13" t="inlineStr">
+      <x:c r="G22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="92" customHeight="1">
-      <x:c r="A22" s="14" t="str">
-        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
-      </x:c>
-      <x:c r="B22" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C22" s="14" t="str">
-        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D22" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E22" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F22" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G22" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="92" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
         <x:v>—</x:v>
@@ -963,347 +971,400 @@
       </x:c>
       <x:c r="F23" s="13" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="13" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="92" customHeight="1">
       <x:c r="A24" s="14" t="str">
+        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+      </x:c>
+      <x:c r="B24" s="18" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="92" customHeight="1">
+      <x:c r="A25" s="13" t="str">
         <x:v>D2.6 — Modello di policy IA di studio e registro degli usi dell'IA</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="str">
+      <x:c r="B25" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
+      <x:c r="C25" s="13" t="str">
         <x:v>I report delle lavorazioni possono alimentare il registro degli usi di Vera. Le scelte per la policy e gli eventuali usi di altri strumenti IA sono forniti dallo studio.</x:v>
       </x:c>
-      <x:c r="D24" s="14" t="str">
+      <x:c r="D25" s="13" t="str">
         <x:v>Implementare il riepilogo degli usi di Vera dai report e la generazione di una bozza di policy IA basata sulle scelte dello studio, integrando gli altri usi dichiarati dallo studio.</x:v>
       </x:c>
-      <x:c r="E24" s="22" t="str">
+      <x:c r="E25" s="21" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F24" s="14" t="inlineStr">
+      <x:c r="F25" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G24" s="14" t="inlineStr">
+      <x:c r="G25" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="25" ht="92" customHeight="1">
-      <x:c r="A25" s="13" t="str">
+    <x:row r="26" ht="92" customHeight="1">
+      <x:c r="A26" s="14" t="str">
         <x:v>D2.7 — Traccia per il registro della formazione/alfabetizzazione IA dei collaboratori</x:v>
       </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="B26" s="18" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
         <x:v>Vera offre corsi guidati sulle proprie funzioni e conserva localmente una traccia delle lezioni, delle esercitazioni e dei progressi dell’utente, utilizzabile per documentare la formazione svolta con Vera.</x:v>
       </x:c>
-      <x:c r="D25" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E25" s="21" t="str">
+      <x:c r="D26" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="str">
         <x:v>Percorso didattico e registrazione locale dei progressi: sorgente locale esaminato
 /Users/fabio/Documents/GitHub/app_files/plugins/vera/skills/learn-with-vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F25" s="13" t="inlineStr">
+      <x:c r="F26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="13" t="inlineStr">
+      <x:c r="G26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="92" customHeight="1">
-      <x:c r="A26" s="14" t="str">
-        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
-      </x:c>
-      <x:c r="B26" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C26" s="14" t="str">
-        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D26" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E26" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F26" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G26" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="27" ht="92" customHeight="1">
       <x:c r="A27" s="13" t="str">
+        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
+      </x:c>
+      <x:c r="B27" s="17" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
+        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D27" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="92" customHeight="1">
+      <x:c r="A28" s="14" t="str">
         <x:v>D2.9 — Testo standard di disclosure sull'uso dell'IA da apporre agli elaborati</x:v>
       </x:c>
-      <x:c r="B27" s="17" t="str">
+      <x:c r="B28" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C27" s="13" t="str">
+      <x:c r="C28" s="14" t="str">
         <x:v>L’inserimento di un testo standard sull’uso dell’IA negli elaborati resta da implementare.</x:v>
       </x:c>
-      <x:c r="D27" s="13" t="str">
+      <x:c r="D28" s="14" t="str">
         <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel.</x:v>
       </x:c>
-      <x:c r="E27" s="21" t="str">
+      <x:c r="E28" s="22" t="str">
         <x:v>Provenienza dei workflow e redazione professionale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F27" s="13" t="inlineStr">
+      <x:c r="F28" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G27" s="13" t="inlineStr">
+      <x:c r="G28" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="92" customHeight="1">
-      <x:c r="A28" s="14" t="str">
-        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
-      </x:c>
-      <x:c r="B28" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C28" s="14" t="str">
-        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D28" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E28" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="29" ht="92" customHeight="1">
       <x:c r="A29" s="13" t="str">
+        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C29" s="13" t="str">
+        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D29" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="92" customHeight="1">
+      <x:c r="A30" s="14" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B29" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C29" s="13" t="str">
+      <x:c r="B30" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
-      <x:c r="D29" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E29" s="21" t="str">
+      <x:c r="D30" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.1
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
-      <x:c r="F29" s="13" t="inlineStr">
+      <x:c r="F30" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G29" s="13" t="inlineStr">
+      <x:c r="G30" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="30" ht="92" customHeight="1">
-      <x:c r="A30" s="14" t="str">
+    <x:row r="31" ht="92" customHeight="1">
+      <x:c r="A31" s="13" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B30" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
         <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E30" s="22" t="str">
+      <x:c r="D31" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E31" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.2
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
-      <x:c r="F30" s="14" t="inlineStr">
+      <x:c r="F31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G30" s="14" t="inlineStr">
+      <x:c r="G31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="31" ht="92" customHeight="1">
-      <x:c r="A31" s="13" t="str">
+    <x:row r="32" ht="92" customHeight="1">
+      <x:c r="A32" s="14" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B31" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
         <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
-      <x:c r="D31" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E31" s="21" t="str">
+      <x:c r="D32" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.3
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
-      <x:c r="F31" s="13" t="inlineStr">
+      <x:c r="F32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
-      <x:c r="G31" s="13" t="inlineStr">
+      <x:c r="G32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="32" ht="92" customHeight="1">
-      <x:c r="A32" s="14" t="str">
+    <x:row r="33" ht="92" customHeight="1">
+      <x:c r="A33" s="13" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B32" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
         <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E32" s="22" t="str">
+      <x:c r="D33" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E33" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.4
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
-      <x:c r="F32" s="14" t="inlineStr">
+      <x:c r="F33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="14" t="inlineStr">
+      <x:c r="G33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="33" ht="92" customHeight="1">
-      <x:c r="A33" s="13" t="str">
+    <x:row r="34" ht="92" customHeight="1">
+      <x:c r="A34" s="14" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B33" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
-      <x:c r="D33" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E33" s="21" t="str">
+      <x:c r="D34" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E34" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.5
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
-      <x:c r="F33" s="13" t="inlineStr">
+      <x:c r="F34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="13" t="inlineStr">
+      <x:c r="G34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="34" ht="92" customHeight="1">
-      <x:c r="A34" s="14" t="str">
+    <x:row r="35" ht="92" customHeight="1">
+      <x:c r="A35" s="15" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B34" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C34" s="14" t="str">
+      <x:c r="B35" s="26" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C35" s="15" t="str">
         <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
-      <x:c r="D34" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E34" s="22" t="str">
+      <x:c r="D35" s="15" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E35" s="23" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.6
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
-      <x:c r="F34" s="14" t="inlineStr">
+      <x:c r="F35" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
-      <x:c r="G34" s="14" t="inlineStr">
+      <x:c r="G35" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="35" ht="92" customHeight="1">
-      <x:c r="A35" s="15" t="str">
+    <x:row r="36" ht="92" customHeight="1">
+      <x:c r="A36" s="3" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B35" s="26" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
+      <x:c r="B36" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
         <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
-      <x:c r="D35" s="15" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="str">
+      <x:c r="D36" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E36" s="29" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.7
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
-      <x:c r="F35" s="15" t="inlineStr">
+      <x:c r="F36" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
-      <x:c r="G35" s="15" t="inlineStr">
+      <x:c r="G36" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">—</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="150" customHeight="1">
+      <x:c r="A37" s="3" t="str">
+        <x:v>N3.8 — Dichiarazione del piano utilizzato all'avvio ed elenco dei presidi che Vera non copre, riportati anche nella documentazione d'uso</x:v>
+      </x:c>
+      <x:c r="B37" s="28" t="str">
+        <x:v>Non previsto</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
+        <x:v>Vera non richiede una dichiarazione del piano utilizzato all’avvio. Le condizioni d’uso pubblicate elencano già i limiti relativi a contratti, account, trattamento dei dati sulla piattaforma e revisione professionale. La scelta del piano resta esterna a Vera, come indicato in G1.6.</x:v>
+      </x:c>
+      <x:c r="D37" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E37" s="29" t="str">
+        <x:v>Condizioni e limiti già pubblicati
+https://mparanza.com/static/shared/vera-compliance/index.html#condizioni-uso
+Piattaforma e piano utilizzato
+https://mparanza.com/static/shared/vera-compliance/index.html#g1-6</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
+        <x:v>Informare lo studio di ciò che resta a suo carico</x:v>
+      </x:c>
+      <x:c r="G37" s="3" t="str">
+        <x:v>Artt. 4 n. 7, 24, 28 GDPR</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1314,7 +1375,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf3644ce8614fb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd233c18d27424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: align Vera compliance assessment with schema 0.2 (#777)
Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rb7d4a3e875584685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdc79cf7a785e4608"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -181,6 +181,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -191,8 +200,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G35"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G37"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Voce dello schema"/>
     <x:tableColumn id="2" name="Stato attuale"/>
@@ -428,9 +437,9 @@
       <x:c r="D2" s="3"/>
       <x:c r="E2" s="3"/>
     </x:row>
-    <x:row r="3" ht="26" customHeight="1">
+    <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>I rapporti con le piattaforme sono trattati come condizioni d’uso. Il connettore di anonimizzazione è opzionale. Base tecnica: sorgente pubblico Vera 0.1.338, 03/10/2026.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026. Riscontro aggiornato al 04/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -778,32 +787,32 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17" ht="92" customHeight="1">
+    <x:row r="17" ht="175" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>G1.12 — Censimento delle skill rispetto all'All. III AI Act e agli artt. 5 e 50, con indicazione di quelle che profilano persone fisiche</x:v>
+        <x:v>G1.12 — Analisi funzione per funzione rispetto all'All. III AI Act e all'art. 6, par. 3, con indicazione di quelle che trattano persone fisiche e producono valutazioni, punteggi o classificazioni</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>Presente</x:v>
+        <x:v>Da implementare</x:v>
       </x:c>
       <x:c r="C17" s="13" t="str">
-        <x:v>Il catalogo descrive le funzioni e i relativi flussi. Nessuna di queste funzioni effettua profilazione di persone fisiche.</x:v>
+        <x:v>Il catalogo descrive le funzioni e i relativi flussi. New Client e la revisione antiriciclaggio trattano anche dati di persone fisiche e includono valutazioni di rischio con revisione professionale. Non è ancora pubblicata l’analisi funzione per funzione richiesta dallo schema 0.2.</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>Documentare, per ciascuna funzione, finalità, persone interessate, valutazioni prodotte e confronto con l’Allegato III e l’art. 6, par. 3. Si tratta di un’analisi da redigere, non di una nuova funzione del software.</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
-        <x:v>Catalogo delle funzioni e degli usi supportati
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/workflow-catalog.md</x:v>
-      </x:c>
-      <x:c r="F17" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Presidiare l'esenzione open source e il rischio di alto rischio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G17" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:t>
-        </x:is>
+        <x:v>Catalogo di Vera
+https://mparanza.com/static/shared/vera/index.html?lang=it#core
+Fascicolo cliente
+https://mparanza.com/static/shared/new-client/index.html?lang=it
+Revisione antiriciclaggio
+https://mparanza.com/static/shared/aml-review/index.html?lang=it</x:v>
+      </x:c>
+      <x:c r="F17" s="13" t="str">
+        <x:v>Presidiare l'esenzione open source e il rischio di alto rischio</x:v>
+      </x:c>
+      <x:c r="G17" s="13" t="str">
+        <x:v>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="92" customHeight="1">
@@ -834,126 +843,125 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="19" ht="92" customHeight="1">
+    <x:row r="19" ht="150" customHeight="1">
       <x:c r="A19" s="13" t="str">
+        <x:v>G1.14 — Marcatura leggibile dalle macchine dei testi generati e rilevabilità come generati artificialmente</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>Non previsto</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str">
+        <x:v>Non è prevista in Vera una funzione dedicata alla marcatura leggibile dalle macchine dei testi generati. L’eventuale marcatura applicata dalla piattaforma AI non è verificata in questo riscontro. La nota visibile sull’uso dell’IA proposta in D2.9 è una funzione distinta.</x:v>
+      </x:c>
+      <x:c r="D19" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E19" s="21" t="str">
+        <x:v>Nota visibile sull’uso dell’IA
+https://mparanza.com/static/shared/vera-compliance/index.html#d2-9
+Art. 50: testo della norma
+https://ai-act-service-desk.ec.europa.eu/en/ai-act/article-50</x:v>
+      </x:c>
+      <x:c r="F19" s="13" t="str">
+        <x:v>Rispettare l'obbligo dei fornitori di sistemi che generano testo sintetico</x:v>
+      </x:c>
+      <x:c r="G19" s="13" t="str">
+        <x:v>Art. 50, par. 2 AI Act; art. 111, par. 4 (Reg. UE 2026/1744)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="92" customHeight="1">
+      <x:c r="A20" s="14" t="str">
         <x:v>D2.1 — Bozza di registro dei trattamenti alimentata dai report di elaborazione</x:v>
       </x:c>
-      <x:c r="B19" s="17" t="str">
+      <x:c r="B20" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C19" s="13" t="str">
+      <x:c r="C20" s="14" t="str">
         <x:v>I report di Vera possono fornire informazioni sulle lavorazioni svolte e sui dati utilizzati.</x:v>
       </x:c>
-      <x:c r="D19" s="13" t="str">
+      <x:c r="D20" s="14" t="str">
         <x:v>Implementare la generazione di una bozza del registro dei trattamenti, integrando i report di Vera con le informazioni fornite dallo studio.</x:v>
       </x:c>
-      <x:c r="E19" s="21" t="str">
+      <x:c r="E20" s="22" t="str">
         <x:v>Report di esecuzione e dati già disponibili
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/model-data-report-contract.md</x:v>
       </x:c>
-      <x:c r="F19" s="13" t="inlineStr">
+      <x:c r="F20" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
-      <x:c r="G19" s="13" t="inlineStr">
+      <x:c r="G20" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="20" ht="92" customHeight="1">
-      <x:c r="A20" s="14" t="str">
+    <x:row r="21" ht="92" customHeight="1">
+      <x:c r="A21" s="13" t="str">
         <x:v>D2.2 — Scheda di screening preliminare per la DPIA</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str">
+      <x:c r="B21" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C21" s="13" t="str">
         <x:v>Vera dispone di percorsi di raccolta delle informazioni e analisi con fonti; la scheda dedicata di screening DPIA resta da implementare.</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="D21" s="13" t="str">
         <x:v>Implementare un percorso guidato che raccolga i fatti sul trattamento, li valuti rispetto ai criteri pertinenti e produca una scheda di screening DPIA motivata, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E20" s="22" t="str">
+      <x:c r="E21" s="21" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F20" s="14" t="inlineStr">
+      <x:c r="F21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G20" s="14" t="inlineStr">
+      <x:c r="G21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21" ht="92" customHeight="1">
-      <x:c r="A21" s="13" t="str">
+    <x:row r="22" ht="92" customHeight="1">
+      <x:c r="A22" s="14" t="str">
         <x:v>D2.3 — Bozza di informativa ai clienti con clausola sull'uso dell'IA</x:v>
       </x:c>
-      <x:c r="B21" s="17" t="str">
+      <x:c r="B22" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C22" s="14" t="str">
         <x:v>New Client raccoglie informazioni privacy/IA e prepara un piano documentale; non produce la bozza dell’informativa richiesta.</x:v>
       </x:c>
-      <x:c r="D21" s="13" t="str">
+      <x:c r="D22" s="14" t="str">
         <x:v>Implementare la generazione di una bozza di informativa ai clienti con clausola sull’uso dell’IA, sulla base delle informazioni dello studio e delle fonti pertinenti, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E21" s="21" t="str">
+      <x:c r="E22" s="22" t="str">
         <x:v>Applicabilità privacy/IA e piano documentale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/new-client/skills/new-client/SKILL.md</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="inlineStr">
+      <x:c r="F22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G21" s="13" t="inlineStr">
+      <x:c r="G22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="92" customHeight="1">
-      <x:c r="A22" s="14" t="str">
-        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
-      </x:c>
-      <x:c r="B22" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C22" s="14" t="str">
-        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D22" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E22" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F22" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G22" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="92" customHeight="1">
       <x:c r="A23" s="13" t="str">
-        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
         <x:v>—</x:v>
@@ -963,347 +971,400 @@
       </x:c>
       <x:c r="F23" s="13" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="13" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="92" customHeight="1">
       <x:c r="A24" s="14" t="str">
+        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+      </x:c>
+      <x:c r="B24" s="18" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E24" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="92" customHeight="1">
+      <x:c r="A25" s="13" t="str">
         <x:v>D2.6 — Modello di policy IA di studio e registro degli usi dell'IA</x:v>
       </x:c>
-      <x:c r="B24" s="18" t="str">
+      <x:c r="B25" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
+      <x:c r="C25" s="13" t="str">
         <x:v>I report delle lavorazioni possono alimentare il registro degli usi di Vera. Le scelte per la policy e gli eventuali usi di altri strumenti IA sono forniti dallo studio.</x:v>
       </x:c>
-      <x:c r="D24" s="14" t="str">
+      <x:c r="D25" s="13" t="str">
         <x:v>Implementare il riepilogo degli usi di Vera dai report e la generazione di una bozza di policy IA basata sulle scelte dello studio, integrando gli altri usi dichiarati dallo studio.</x:v>
       </x:c>
-      <x:c r="E24" s="22" t="str">
+      <x:c r="E25" s="21" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F24" s="14" t="inlineStr">
+      <x:c r="F25" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G24" s="14" t="inlineStr">
+      <x:c r="G25" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="25" ht="92" customHeight="1">
-      <x:c r="A25" s="13" t="str">
+    <x:row r="26" ht="92" customHeight="1">
+      <x:c r="A26" s="14" t="str">
         <x:v>D2.7 — Traccia per il registro della formazione/alfabetizzazione IA dei collaboratori</x:v>
       </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="B26" s="18" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
         <x:v>Vera offre corsi guidati sulle proprie funzioni e conserva localmente una traccia delle lezioni, delle esercitazioni e dei progressi dell’utente, utilizzabile per documentare la formazione svolta con Vera.</x:v>
       </x:c>
-      <x:c r="D25" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E25" s="21" t="str">
+      <x:c r="D26" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E26" s="22" t="str">
         <x:v>Percorso didattico e registrazione locale dei progressi: sorgente locale esaminato
 /Users/fabio/Documents/GitHub/app_files/plugins/vera/skills/learn-with-vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F25" s="13" t="inlineStr">
+      <x:c r="F26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="13" t="inlineStr">
+      <x:c r="G26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="92" customHeight="1">
-      <x:c r="A26" s="14" t="str">
-        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
-      </x:c>
-      <x:c r="B26" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C26" s="14" t="str">
-        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D26" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E26" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F26" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G26" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="27" ht="92" customHeight="1">
       <x:c r="A27" s="13" t="str">
+        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
+      </x:c>
+      <x:c r="B27" s="17" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
+        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D27" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F27" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="92" customHeight="1">
+      <x:c r="A28" s="14" t="str">
         <x:v>D2.9 — Testo standard di disclosure sull'uso dell'IA da apporre agli elaborati</x:v>
       </x:c>
-      <x:c r="B27" s="17" t="str">
+      <x:c r="B28" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C27" s="13" t="str">
+      <x:c r="C28" s="14" t="str">
         <x:v>L’inserimento di un testo standard sull’uso dell’IA negli elaborati resta da implementare.</x:v>
       </x:c>
-      <x:c r="D27" s="13" t="str">
+      <x:c r="D28" s="14" t="str">
         <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel.</x:v>
       </x:c>
-      <x:c r="E27" s="21" t="str">
+      <x:c r="E28" s="22" t="str">
         <x:v>Provenienza dei workflow e redazione professionale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F27" s="13" t="inlineStr">
+      <x:c r="F28" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G27" s="13" t="inlineStr">
+      <x:c r="G28" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="92" customHeight="1">
-      <x:c r="A28" s="14" t="str">
-        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
-      </x:c>
-      <x:c r="B28" s="18" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C28" s="14" t="str">
-        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D28" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E28" s="22" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="29" ht="92" customHeight="1">
       <x:c r="A29" s="13" t="str">
+        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C29" s="13" t="str">
+        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D29" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F29" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="92" customHeight="1">
+      <x:c r="A30" s="14" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B29" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C29" s="13" t="str">
+      <x:c r="B30" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
-      <x:c r="D29" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E29" s="21" t="str">
+      <x:c r="D30" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.1
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
-      <x:c r="F29" s="13" t="inlineStr">
+      <x:c r="F30" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G29" s="13" t="inlineStr">
+      <x:c r="G30" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="30" ht="92" customHeight="1">
-      <x:c r="A30" s="14" t="str">
+    <x:row r="31" ht="92" customHeight="1">
+      <x:c r="A31" s="13" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B30" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
         <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E30" s="22" t="str">
+      <x:c r="D31" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E31" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.2
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
-      <x:c r="F30" s="14" t="inlineStr">
+      <x:c r="F31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G30" s="14" t="inlineStr">
+      <x:c r="G31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="31" ht="92" customHeight="1">
-      <x:c r="A31" s="13" t="str">
+    <x:row r="32" ht="92" customHeight="1">
+      <x:c r="A32" s="14" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B31" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
         <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
-      <x:c r="D31" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E31" s="21" t="str">
+      <x:c r="D32" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.3
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
-      <x:c r="F31" s="13" t="inlineStr">
+      <x:c r="F32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
-      <x:c r="G31" s="13" t="inlineStr">
+      <x:c r="G32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="32" ht="92" customHeight="1">
-      <x:c r="A32" s="14" t="str">
+    <x:row r="33" ht="92" customHeight="1">
+      <x:c r="A33" s="13" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B32" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
         <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E32" s="22" t="str">
+      <x:c r="D33" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E33" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.4
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
-      <x:c r="F32" s="14" t="inlineStr">
+      <x:c r="F33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="14" t="inlineStr">
+      <x:c r="G33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="33" ht="92" customHeight="1">
-      <x:c r="A33" s="13" t="str">
+    <x:row r="34" ht="92" customHeight="1">
+      <x:c r="A34" s="14" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B33" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
-      <x:c r="D33" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E33" s="21" t="str">
+      <x:c r="D34" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E34" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.5
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
-      <x:c r="F33" s="13" t="inlineStr">
+      <x:c r="F34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="13" t="inlineStr">
+      <x:c r="G34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="34" ht="92" customHeight="1">
-      <x:c r="A34" s="14" t="str">
+    <x:row r="35" ht="92" customHeight="1">
+      <x:c r="A35" s="15" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B34" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C34" s="14" t="str">
+      <x:c r="B35" s="26" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C35" s="15" t="str">
         <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
-      <x:c r="D34" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E34" s="22" t="str">
+      <x:c r="D35" s="15" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E35" s="23" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.6
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
-      <x:c r="F34" s="14" t="inlineStr">
+      <x:c r="F35" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
-      <x:c r="G34" s="14" t="inlineStr">
+      <x:c r="G35" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="35" ht="92" customHeight="1">
-      <x:c r="A35" s="15" t="str">
+    <x:row r="36" ht="92" customHeight="1">
+      <x:c r="A36" s="3" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B35" s="26" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
+      <x:c r="B36" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C36" s="3" t="str">
         <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
-      <x:c r="D35" s="15" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="str">
+      <x:c r="D36" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E36" s="29" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.7
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
-      <x:c r="F35" s="15" t="inlineStr">
+      <x:c r="F36" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
-      <x:c r="G35" s="15" t="inlineStr">
+      <x:c r="G36" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">—</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="150" customHeight="1">
+      <x:c r="A37" s="3" t="str">
+        <x:v>N3.8 — Dichiarazione del piano utilizzato all'avvio ed elenco dei presidi che Vera non copre, riportati anche nella documentazione d'uso</x:v>
+      </x:c>
+      <x:c r="B37" s="28" t="str">
+        <x:v>Non previsto</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
+        <x:v>Vera non richiede una dichiarazione del piano utilizzato all’avvio. Le condizioni d’uso pubblicate elencano già i limiti relativi a contratti, account, trattamento dei dati sulla piattaforma e revisione professionale. La scelta del piano resta esterna a Vera, come indicato in G1.6.</x:v>
+      </x:c>
+      <x:c r="D37" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E37" s="29" t="str">
+        <x:v>Condizioni e limiti già pubblicati
+https://mparanza.com/static/shared/vera-compliance/index.html#condizioni-uso
+Piattaforma e piano utilizzato
+https://mparanza.com/static/shared/vera-compliance/index.html#g1-6</x:v>
+      </x:c>
+      <x:c r="F37" s="3" t="str">
+        <x:v>Informare lo studio di ciò che resta a suo carico</x:v>
+      </x:c>
+      <x:c r="G37" s="3" t="str">
+        <x:v>Artt. 4 n. 7, 24, 28 GDPR</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1314,7 +1375,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf3644ce8614fb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd233c18d27424f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: align Vera compliance correspondence and public disclosures
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdc79cf7a785e4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Ra36cc176fb9649f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -190,6 +190,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -200,8 +209,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G37"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G39"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Voce dello schema"/>
     <x:tableColumn id="2" name="Stato attuale"/>
@@ -439,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026. Riscontro aggiornato al 04/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 07/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -564,7 +573,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="92" customHeight="1">
+    <x:row r="9" ht="409.5" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>G1.4 — Collegamento in input con motore di anonimizzazione, con descrizione della tecnica e conservazione locale della tabella di corrispondenza</x:v>
       </x:c>
@@ -572,14 +581,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>Vera dispone di collegamenti opzionali a motori di anonimizzazione e utilizza il risultato restituito dal connettore. La tecnica e la gestione dell’eventuale mappa di corrispondenza dipendono dal motore e dall’integrazione scelti.</x:v>
+        <x:v>Vera offre collegamenti opzionali a cinque motori di anonimizzazione con caratteristiche diverse: OpenAI Privacy Filter, GLiNER2-PII, Rizzo PII, Lethe e PII-Shield. La scelta del motore spetta all’utente; al momento Mparanza non ne raccomanda uno.
+Non tutti sono adatti ai lavori AI che devono riconoscere lo stesso soggetto in documenti diversi. Fra i cinque elencati, solo i percorsi descritti per Lethe e PII-Shield prevedono segnaposto coerenti tra più documenti dello stesso lavoro. La sola rimozione degli identificativi non conserva necessariamente queste relazioni.
+L’elenco riporta indicazioni tratte dalla documentazione dei rispettivi autori. Le caratteristiche e l’efficacia dichiarate non sono state validate da Mparanza per l’uso professionale dello studio.</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>Siamo consapevoli che dover scegliere e valutare il motore non è una soluzione attrattiva per un piccolo studio. In futuro ci proponiamo di individuare e consigliare soluzioni più efficaci, quando avremo elementi per indicarle.</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>Connettori locali opzionali: contratto operativo
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/optional-integrations.md</x:v>
+        <x:v>Indicazioni degli autori, non validate da Mparanza per l’uso professionale.
+OpenAI Privacy Filter: Rileva e maschera identificativi; non descrive un dizionario reversibile tra documenti.
+GLiNER2-PII: Rileva entità; l’esempio usa etichette di categoria, senza identità condivise tra documenti.
+Rizzo PII: Segnaposto e dizionario locale reversibile; continuità tra elaborazioni separate non documentata.
+Lethe: Dizionario e segnaposto stabili per un lavoro su più file; ripristino dei valori.
+PII-Shield: Sessioni tra più documenti, segnaposto condivisi e ripristino dei valori.
+Elenco, fonti e istruzioni:
+https://mparanza.com/static/shared/vera-compliance/index.html#motori-anonimizzazione</x:v>
       </x:c>
       <x:c r="F9" s="13" t="inlineStr">
         <x:is>
@@ -592,7 +609,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="92" customHeight="1">
+    <x:row r="10" ht="409.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>G1.5 — Assenza di telemetria e di invio di dati agli sviluppatori per impostazione predefinita (eventuale opt-in documentato)</x:v>
       </x:c>
@@ -600,14 +617,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>Documenti e contenuti del fascicolo non vengono inviati a Mparanza. Il servizio riceve una ricevuta tecnica, senza tali contenuti; anche le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
+        <x:v>Il report resta locale. Vera ne calcola l’hash SHA-256: un’impronta di 64 caratteri, non una copia cifrata. Invia automaticamente hash, versione dello schema, ID casuale della ricevuta e versione di Vera. Non invia report, documenti, nomi dei file, prompt o output del modello. La verifica confronta l’hash ricalcolato localmente con la prova firmata (N3.9).
+Mparanza non riceve nomi dei clienti né una corrispondenza fra hash e persone. L’ID identifica la ricevuta. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo (considerando 26): l’invio crea la prova tecnica senza comunicare i contenuti.
+Il servizio opera e conserva le ricevute in Finlandia (UE); Mparanza LLC è costituita in Delaware.
+L’IP non serve alla ricevuta e non è salvato nel suo database. L’endpoint lo usa per limitare richieste eccessive; i log degli accessi lo registrano separatamente.
+Nginx conserva 14 archivi giornalieri più il corrente. Per il log Uvicorn non risulta un termine massimo; lo script lo sovrascrive al riavvio.
+La prova firmata è conservata senza scadenza automatica. Le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>—</x:v>
+        <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
         <x:v>build_receipt_request(): quattro campi ammessi
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py</x:v>
+https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py
+Configurazione e log del server verificati il 07/10/2026.
+Conservazione della prova firmata: modules/run_receipts/store.py, schema e metodi stamp()/get(), verificati il 07/10/2026.
+Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -798,7 +823,7 @@
         <x:v>Il catalogo descrive le funzioni e i relativi flussi. New Client e la revisione antiriciclaggio trattano anche dati di persone fisiche e includono valutazioni di rischio con revisione professionale. Non è ancora pubblicata l’analisi funzione per funzione richiesta dallo schema 0.2.</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>Documentare, per ciascuna funzione, finalità, persone interessate, valutazioni prodotte e confronto con l’Allegato III e l’art. 6, par. 3. Si tratta di un’analisi da redigere, non di una nuova funzione del software.</x:v>
+        <x:v>Compilare una griglia partendo dalle descrizioni dei processi di Vera: finalità prevista, persone interessate, valutazioni o punteggi prodotti, confronto con l’Allegato III e gli artt. 5, 6 e 50 AI Act, separabilità dalle altre funzioni. Approfondire le qualificazioni normative che lo richiedono. Il lavoro da completare è questa analisi documentata delle funzioni esistenti.</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
         <x:v>Catalogo di Vera
@@ -815,7 +840,7 @@
         <x:v>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="92" customHeight="1">
+    <x:row r="18" ht="225" customHeight="1">
       <x:c r="A18" s="14" t="str">
         <x:v>G1.13 — Versionamento, registro delle modifiche e indicazione della licenza</x:v>
       </x:c>
@@ -823,14 +848,17 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.</x:v>
+        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.
+Abbiamo considerato la possibilità di offrire a pagamento il servizio server di attestazione tecnica dei report e non la escludiamo. Allo stato riteniamo però che, per gran parte degli utilizzatori, un servizio aggiuntivo di questo tipo possa risultare largamente ridondante: Vera è open source e il suo funzionamento, compresi elaborazione locale e minimizzazione dei dati, è documentato e verificabile. Questa è la nostra valutazione della sua utilità commerciale. L’eventuale attestazione avrebbe per oggetto l’esistenza e l’integrità del report.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="E18" s="22" t="str">
-        <x:v>Manifest Vera 0.1.338, repository e AGPL-3.0-only
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/.codex-plugin/plugin.json</x:v>
+        <x:v>Manifest corrente di Vera, repository e AGPL-3.0-only
+https://github.com/fabioannovazzi/app_files/blob/main/plugins/vera/.codex-plugin/plugin.json
+Licenza, servizi e modello economico: valutazione commerciale di Mparanza aggiornata al 07/10/2026.
+https://mparanza.com/static/shared/vera-compliance/index.html#attestazione-servizio</x:v>
       </x:c>
       <x:c r="F18" s="14" t="inlineStr">
         <x:is>
@@ -869,126 +897,125 @@
         <x:v>Art. 50, par. 2 AI Act; art. 111, par. 4 (Reg. UE 2026/1744)</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="92" customHeight="1">
+    <x:row r="20" ht="220" customHeight="1">
       <x:c r="A20" s="14" t="str">
+        <x:v>G1.15 — Descrizione unica e coerente delle funzioni e dei limiti d’uso in documentazione, termini d’uso e comunicazione pubblica</x:v>
+      </x:c>
+      <x:c r="B20" s="18" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12.</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="str">
+        <x:v>Funzioni e limiti d’uso: https://mparanza.com/terms#vera-functions-and-limits
+Ricevute: https://mparanza.com/zero-retention#run-receipts
+Catalogo: https://mparanza.com/static/shared/vera/index.html?lang=it
+Integrazioni: https://mparanza.com/static/shared/vera-integrazioni/index.html</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>Coerenza della descrizione delle funzioni e dei limiti d’uso fra documentazione, termini e comunicazione pubblica.</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>Art. 3, punto 12 AI Act; documento di orientamento della Commissione, parr. 10-14 (riferimenti dello schema di osservazioni).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="92" customHeight="1">
+      <x:c r="A21" s="13" t="str">
         <x:v>D2.1 — Bozza di registro dei trattamenti alimentata dai report di elaborazione</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str">
+      <x:c r="B21" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C21" s="13" t="str">
         <x:v>I report di Vera possono fornire informazioni sulle lavorazioni svolte e sui dati utilizzati.</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="D21" s="13" t="str">
         <x:v>Implementare la generazione di una bozza del registro dei trattamenti, integrando i report di Vera con le informazioni fornite dallo studio.</x:v>
       </x:c>
-      <x:c r="E20" s="22" t="str">
+      <x:c r="E21" s="21" t="str">
         <x:v>Report di esecuzione e dati già disponibili
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/model-data-report-contract.md</x:v>
       </x:c>
-      <x:c r="F20" s="14" t="inlineStr">
+      <x:c r="F21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
-      <x:c r="G20" s="14" t="inlineStr">
+      <x:c r="G21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21" ht="92" customHeight="1">
-      <x:c r="A21" s="13" t="str">
+    <x:row r="22" ht="92" customHeight="1">
+      <x:c r="A22" s="14" t="str">
         <x:v>D2.2 — Scheda di screening preliminare per la DPIA</x:v>
       </x:c>
-      <x:c r="B21" s="17" t="str">
+      <x:c r="B22" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C22" s="14" t="str">
         <x:v>Vera dispone di percorsi di raccolta delle informazioni e analisi con fonti; la scheda dedicata di screening DPIA resta da implementare.</x:v>
       </x:c>
-      <x:c r="D21" s="13" t="str">
+      <x:c r="D22" s="14" t="str">
         <x:v>Implementare un percorso guidato che raccolga i fatti sul trattamento, li valuti rispetto ai criteri pertinenti e produca una scheda di screening DPIA motivata, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E21" s="21" t="str">
+      <x:c r="E22" s="22" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="inlineStr">
+      <x:c r="F22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G21" s="13" t="inlineStr">
+      <x:c r="G22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="22" ht="92" customHeight="1">
-      <x:c r="A22" s="14" t="str">
+    <x:row r="23" ht="92" customHeight="1">
+      <x:c r="A23" s="13" t="str">
         <x:v>D2.3 — Bozza di informativa ai clienti con clausola sull'uso dell'IA</x:v>
       </x:c>
-      <x:c r="B22" s="18" t="str">
+      <x:c r="B23" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C22" s="14" t="str">
+      <x:c r="C23" s="13" t="str">
         <x:v>New Client raccoglie informazioni privacy/IA e prepara un piano documentale; non produce la bozza dell’informativa richiesta.</x:v>
       </x:c>
-      <x:c r="D22" s="14" t="str">
+      <x:c r="D23" s="13" t="str">
         <x:v>Implementare la generazione di una bozza di informativa ai clienti con clausola sull’uso dell’IA, sulla base delle informazioni dello studio e delle fonti pertinenti, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E22" s="22" t="str">
+      <x:c r="E23" s="21" t="str">
         <x:v>Applicabilità privacy/IA e piano documentale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/new-client/skills/new-client/SKILL.md</x:v>
       </x:c>
-      <x:c r="F22" s="14" t="inlineStr">
+      <x:c r="F23" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G22" s="14" t="inlineStr">
+      <x:c r="G23" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="92" customHeight="1">
-      <x:c r="A23" s="13" t="str">
-        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
-      </x:c>
-      <x:c r="B23" s="17" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C23" s="13" t="str">
-        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D23" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E23" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F23" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G23" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="92" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
       </x:c>
       <x:c r="B24" s="18" t="str">
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
         <x:v>—</x:v>
@@ -998,373 +1025,433 @@
       </x:c>
       <x:c r="F24" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="25" ht="92" customHeight="1">
       <x:c r="A25" s="13" t="str">
+        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E25" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="92" customHeight="1">
+      <x:c r="A26" s="14" t="str">
         <x:v>D2.6 — Modello di policy IA di studio e registro degli usi dell'IA</x:v>
       </x:c>
-      <x:c r="B25" s="17" t="str">
+      <x:c r="B26" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="C26" s="14" t="str">
         <x:v>I report delle lavorazioni possono alimentare il registro degli usi di Vera. Le scelte per la policy e gli eventuali usi di altri strumenti IA sono forniti dallo studio.</x:v>
       </x:c>
-      <x:c r="D25" s="13" t="str">
+      <x:c r="D26" s="14" t="str">
         <x:v>Implementare il riepilogo degli usi di Vera dai report e la generazione di una bozza di policy IA basata sulle scelte dello studio, integrando gli altri usi dichiarati dallo studio.</x:v>
       </x:c>
-      <x:c r="E25" s="21" t="str">
+      <x:c r="E26" s="22" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F25" s="13" t="inlineStr">
+      <x:c r="F26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="13" t="inlineStr">
+      <x:c r="G26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="26" ht="92" customHeight="1">
-      <x:c r="A26" s="14" t="str">
+    <x:row r="27" ht="92" customHeight="1">
+      <x:c r="A27" s="13" t="str">
         <x:v>D2.7 — Traccia per il registro della formazione/alfabetizzazione IA dei collaboratori</x:v>
       </x:c>
-      <x:c r="B26" s="18" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C26" s="14" t="str">
+      <x:c r="B27" s="17" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
         <x:v>Vera offre corsi guidati sulle proprie funzioni e conserva localmente una traccia delle lezioni, delle esercitazioni e dei progressi dell’utente, utilizzabile per documentare la formazione svolta con Vera.</x:v>
       </x:c>
-      <x:c r="D26" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E26" s="22" t="str">
+      <x:c r="D27" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
         <x:v>Percorso didattico e registrazione locale dei progressi: sorgente locale esaminato
 /Users/fabio/Documents/GitHub/app_files/plugins/vera/skills/learn-with-vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F26" s="14" t="inlineStr">
+      <x:c r="F27" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
-      <x:c r="G26" s="14" t="inlineStr">
+      <x:c r="G27" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="92" customHeight="1">
-      <x:c r="A27" s="13" t="str">
-        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
-      </x:c>
-      <x:c r="B27" s="17" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C27" s="13" t="str">
-        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D27" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E27" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F27" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G27" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="28" ht="92" customHeight="1">
       <x:c r="A28" s="14" t="str">
+        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E28" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="135" customHeight="1">
+      <x:c r="A29" s="13" t="str">
         <x:v>D2.9 — Testo standard di disclosure sull'uso dell'IA da apporre agli elaborati</x:v>
       </x:c>
-      <x:c r="B28" s="18" t="str">
+      <x:c r="B29" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C28" s="14" t="str">
+      <x:c r="C29" s="13" t="str">
         <x:v>L’inserimento di un testo standard sull’uso dell’IA negli elaborati resta da implementare.</x:v>
       </x:c>
-      <x:c r="D28" s="14" t="str">
-        <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel.</x:v>
-      </x:c>
-      <x:c r="E28" s="22" t="str">
+      <x:c r="D29" s="13" t="str">
+        <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel. Da decidere: inserimento automatico per impostazione predefinita e possibilità per lo studio di modificarne il testo.</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
         <x:v>Provenienza dei workflow e redazione professionale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F28" s="14" t="inlineStr">
+      <x:c r="F29" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G28" s="14" t="inlineStr">
+      <x:c r="G29" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="92" customHeight="1">
-      <x:c r="A29" s="13" t="str">
-        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
-      </x:c>
-      <x:c r="B29" s="24" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C29" s="13" t="str">
-        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D29" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E29" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F29" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G29" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="30" ht="92" customHeight="1">
       <x:c r="A30" s="14" t="str">
+        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
+      </x:c>
+      <x:c r="B30" s="25" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="92" customHeight="1">
+      <x:c r="A31" s="13" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B30" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E30" s="22" t="str">
+      <x:c r="D31" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E31" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.1
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
-      <x:c r="F30" s="14" t="inlineStr">
+      <x:c r="F31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G30" s="14" t="inlineStr">
+      <x:c r="G31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="31" ht="92" customHeight="1">
-      <x:c r="A31" s="13" t="str">
+    <x:row r="32" ht="92" customHeight="1">
+      <x:c r="A32" s="14" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B31" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
         <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
-      <x:c r="D31" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E31" s="21" t="str">
+      <x:c r="D32" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.2
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
-      <x:c r="F31" s="13" t="inlineStr">
+      <x:c r="F32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G31" s="13" t="inlineStr">
+      <x:c r="G32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="32" ht="92" customHeight="1">
-      <x:c r="A32" s="14" t="str">
+    <x:row r="33" ht="92" customHeight="1">
+      <x:c r="A33" s="13" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B32" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
         <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E32" s="22" t="str">
+      <x:c r="D33" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E33" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.3
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
-      <x:c r="F32" s="14" t="inlineStr">
+      <x:c r="F33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="14" t="inlineStr">
+      <x:c r="G33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="33" ht="92" customHeight="1">
-      <x:c r="A33" s="13" t="str">
+    <x:row r="34" ht="92" customHeight="1">
+      <x:c r="A34" s="14" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B33" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
         <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
-      <x:c r="D33" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E33" s="21" t="str">
+      <x:c r="D34" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E34" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.4
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
-      <x:c r="F33" s="13" t="inlineStr">
+      <x:c r="F34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="13" t="inlineStr">
+      <x:c r="G34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="34" ht="92" customHeight="1">
-      <x:c r="A34" s="14" t="str">
+    <x:row r="35" ht="92" customHeight="1">
+      <x:c r="A35" s="13" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B34" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C34" s="14" t="str">
+      <x:c r="B35" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
-      <x:c r="D34" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E34" s="22" t="str">
+      <x:c r="D35" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E35" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.5
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
-      <x:c r="F34" s="14" t="inlineStr">
+      <x:c r="F35" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G34" s="14" t="inlineStr">
+      <x:c r="G35" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="35" ht="92" customHeight="1">
-      <x:c r="A35" s="15" t="str">
+    <x:row r="36" ht="92" customHeight="1">
+      <x:c r="A36" s="11" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B35" s="26" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
+      <x:c r="B36" s="31" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="str">
         <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
-      <x:c r="D35" s="15" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="str">
+      <x:c r="D36" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E36" s="32" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.6
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
-      <x:c r="F35" s="15" t="inlineStr">
+      <x:c r="F36" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
-      <x:c r="G35" s="15" t="inlineStr">
+      <x:c r="G36" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="36" ht="92" customHeight="1">
-      <x:c r="A36" s="3" t="str">
+    <x:row r="37" ht="92" customHeight="1">
+      <x:c r="A37" s="3" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B36" s="28" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C36" s="3" t="str">
+      <x:c r="B37" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
         <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
-      <x:c r="D36" s="3" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E36" s="29" t="str">
+      <x:c r="D37" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E37" s="29" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.7
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
-      <x:c r="F36" s="3" t="inlineStr">
+      <x:c r="F37" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
-      <x:c r="G36" s="3" t="inlineStr">
+      <x:c r="G37" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="37" ht="150" customHeight="1">
-      <x:c r="A37" s="3" t="str">
+    <x:row r="38" ht="150" customHeight="1">
+      <x:c r="A38" s="3" t="str">
         <x:v>N3.8 — Dichiarazione del piano utilizzato all'avvio ed elenco dei presidi che Vera non copre, riportati anche nella documentazione d'uso</x:v>
       </x:c>
-      <x:c r="B37" s="28" t="str">
+      <x:c r="B38" s="28" t="str">
         <x:v>Non previsto</x:v>
       </x:c>
-      <x:c r="C37" s="3" t="str">
+      <x:c r="C38" s="3" t="str">
         <x:v>Vera non richiede una dichiarazione del piano utilizzato all’avvio. Le condizioni d’uso pubblicate elencano già i limiti relativi a contratti, account, trattamento dei dati sulla piattaforma e revisione professionale. La scelta del piano resta esterna a Vera, come indicato in G1.6.</x:v>
       </x:c>
-      <x:c r="D37" s="3" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E37" s="29" t="str">
+      <x:c r="D38" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E38" s="29" t="str">
         <x:v>Condizioni e limiti già pubblicati
 https://mparanza.com/static/shared/vera-compliance/index.html#condizioni-uso
 Piattaforma e piano utilizzato
 https://mparanza.com/static/shared/vera-compliance/index.html#g1-6</x:v>
       </x:c>
-      <x:c r="F37" s="3" t="str">
+      <x:c r="F38" s="3" t="str">
         <x:v>Informare lo studio di ciò che resta a suo carico</x:v>
       </x:c>
-      <x:c r="G37" s="3" t="str">
+      <x:c r="G38" s="3" t="str">
         <x:v>Artt. 4 n. 7, 24, 28 GDPR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="405" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>N3.9 — Dichiarazione sul servizio delle ricevute tecniche</x:v>
+      </x:c>
+      <x:c r="B39" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>Vera calcola sul computer l’hash SHA-256 del report: una stringa di 64 caratteri. È un’impronta per confrontare documenti, non una copia cifrata del report: non esiste un’operazione di decifratura che ne restituisca il contenuto.
+Il comando che genera il report con ricevuta invia automaticamente solo quell’impronta, la versione dello schema, un ID casuale della ricevuta e la versione di Vera. Non invia report, documenti del cliente, nomi dei file, prompt o risposte del modello.
+Mparanza firma la prova con la data del server. Chi possiede il report può ricalcolarne l’hash sul proprio computer e confrontarlo con la prova firmata: la verifica non richiede l’invio del report a Mparanza. Il servizio opera in Finlandia e conserva la prova senza scadenza automatica.
+Mparanza non riceve nomi o identificativi dei clienti né la corrispondenza fra hash e persone. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo. Non prevediamo un interruttore per disattivare l’invio della ricevuta: non aggiungerebbe protezione ai contenuti del fascicolo, che non vengono trasmessi. L’invio automatico crea la prova tecnica. I log di connessione sono distinti e descritti separatamente.</x:v>
+      </x:c>
+      <x:c r="D39" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E39" s="29" t="str">
+        <x:v>Dichiarazione N3.9
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-9
+Descrizione del servizio e dei log
+https://mparanza.com/zero-retention#run-receipts
+Log distinti dalle ricevute: IP, URL ed esito HTTP. L’URL può includere ID della ricevuta e hash; non contiene report o documenti. L’IP serve a limitare richieste eccessive e non è nel database delle ricevute.
+Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.
+Mparanza LLC opera come titolare autonomo per i log tecnici del proprio servizio, con finalità di sicurezza e prevenzione degli abusi. La base giuridica individuata è il legittimo interesse (art. 6, par. 1, lett. f, GDPR), nei limiti di necessità e proporzionalità. Referente e rappresentante di Mparanza LLC: Fabio Annovazzi, Anières (Svizzera).
+Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>Descrivere agli studi il funzionamento e i dati del servizio di ricevuta tecnica.</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
+        <x:v>Artt. 13, 28 GDPR (riferimenti indicati nello schema di osservazioni).</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1375,7 +1462,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd233c18d27424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re99f4807f93640c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: align Vera compliance correspondence and public disclosures (#792)
* docs: align Vera compliance correspondence and public disclosures

* chore: refresh privacy review bindings for shared legal copy

---------

Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdc79cf7a785e4608"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Ra36cc176fb9649f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -105,7 +105,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -190,6 +190,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -200,8 +209,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:G37"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RiscontroNicola" displayName="RiscontroNicola" ref="A5:G39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:G39"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Voce dello schema"/>
     <x:tableColumn id="2" name="Stato attuale"/>
@@ -439,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026. Riscontro aggiornato al 04/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 07/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -564,7 +573,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="9" ht="92" customHeight="1">
+    <x:row r="9" ht="409.5" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>G1.4 — Collegamento in input con motore di anonimizzazione, con descrizione della tecnica e conservazione locale della tabella di corrispondenza</x:v>
       </x:c>
@@ -572,14 +581,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C9" s="13" t="str">
-        <x:v>Vera dispone di collegamenti opzionali a motori di anonimizzazione e utilizza il risultato restituito dal connettore. La tecnica e la gestione dell’eventuale mappa di corrispondenza dipendono dal motore e dall’integrazione scelti.</x:v>
+        <x:v>Vera offre collegamenti opzionali a cinque motori di anonimizzazione con caratteristiche diverse: OpenAI Privacy Filter, GLiNER2-PII, Rizzo PII, Lethe e PII-Shield. La scelta del motore spetta all’utente; al momento Mparanza non ne raccomanda uno.
+Non tutti sono adatti ai lavori AI che devono riconoscere lo stesso soggetto in documenti diversi. Fra i cinque elencati, solo i percorsi descritti per Lethe e PII-Shield prevedono segnaposto coerenti tra più documenti dello stesso lavoro. La sola rimozione degli identificativi non conserva necessariamente queste relazioni.
+L’elenco riporta indicazioni tratte dalla documentazione dei rispettivi autori. Le caratteristiche e l’efficacia dichiarate non sono state validate da Mparanza per l’uso professionale dello studio.</x:v>
       </x:c>
       <x:c r="D9" s="13" t="str">
-        <x:v>—</x:v>
+        <x:v>Siamo consapevoli che dover scegliere e valutare il motore non è una soluzione attrattiva per un piccolo studio. In futuro ci proponiamo di individuare e consigliare soluzioni più efficaci, quando avremo elementi per indicarle.</x:v>
       </x:c>
       <x:c r="E9" s="21" t="str">
-        <x:v>Connettori locali opzionali: contratto operativo
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/optional-integrations.md</x:v>
+        <x:v>Indicazioni degli autori, non validate da Mparanza per l’uso professionale.
+OpenAI Privacy Filter: Rileva e maschera identificativi; non descrive un dizionario reversibile tra documenti.
+GLiNER2-PII: Rileva entità; l’esempio usa etichette di categoria, senza identità condivise tra documenti.
+Rizzo PII: Segnaposto e dizionario locale reversibile; continuità tra elaborazioni separate non documentata.
+Lethe: Dizionario e segnaposto stabili per un lavoro su più file; ripristino dei valori.
+PII-Shield: Sessioni tra più documenti, segnaposto condivisi e ripristino dei valori.
+Elenco, fonti e istruzioni:
+https://mparanza.com/static/shared/vera-compliance/index.html#motori-anonimizzazione</x:v>
       </x:c>
       <x:c r="F9" s="13" t="inlineStr">
         <x:is>
@@ -592,7 +609,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="10" ht="92" customHeight="1">
+    <x:row r="10" ht="409.5" customHeight="1">
       <x:c r="A10" s="14" t="str">
         <x:v>G1.5 — Assenza di telemetria e di invio di dati agli sviluppatori per impostazione predefinita (eventuale opt-in documentato)</x:v>
       </x:c>
@@ -600,14 +617,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>Documenti e contenuti del fascicolo non vengono inviati a Mparanza. Il servizio riceve una ricevuta tecnica, senza tali contenuti; anche le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
+        <x:v>Il report resta locale. Vera ne calcola l’hash SHA-256: un’impronta di 64 caratteri, non una copia cifrata. Invia automaticamente hash, versione dello schema, ID casuale della ricevuta e versione di Vera. Non invia report, documenti, nomi dei file, prompt o output del modello. La verifica confronta l’hash ricalcolato localmente con la prova firmata (N3.9).
+Mparanza non riceve nomi dei clienti né una corrispondenza fra hash e persone. L’ID identifica la ricevuta. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo (considerando 26): l’invio crea la prova tecnica senza comunicare i contenuti.
+Il servizio opera e conserva le ricevute in Finlandia (UE); Mparanza LLC è costituita in Delaware.
+L’IP non serve alla ricevuta e non è salvato nel suo database. L’endpoint lo usa per limitare richieste eccessive; i log degli accessi lo registrano separatamente.
+Nginx conserva 14 archivi giornalieri più il corrente. Per il log Uvicorn non risulta un termine massimo; lo script lo sovrascrive al riavvio.
+La prova firmata è conservata senza scadenza automatica. Le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
-        <x:v>—</x:v>
+        <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
         <x:v>build_receipt_request(): quattro campi ammessi
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py</x:v>
+https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py
+Configurazione e log del server verificati il 07/10/2026.
+Conservazione della prova firmata: modules/run_receipts/store.py, schema e metodi stamp()/get(), verificati il 07/10/2026.
+Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -798,7 +823,7 @@
         <x:v>Il catalogo descrive le funzioni e i relativi flussi. New Client e la revisione antiriciclaggio trattano anche dati di persone fisiche e includono valutazioni di rischio con revisione professionale. Non è ancora pubblicata l’analisi funzione per funzione richiesta dallo schema 0.2.</x:v>
       </x:c>
       <x:c r="D17" s="13" t="str">
-        <x:v>Documentare, per ciascuna funzione, finalità, persone interessate, valutazioni prodotte e confronto con l’Allegato III e l’art. 6, par. 3. Si tratta di un’analisi da redigere, non di una nuova funzione del software.</x:v>
+        <x:v>Compilare una griglia partendo dalle descrizioni dei processi di Vera: finalità prevista, persone interessate, valutazioni o punteggi prodotti, confronto con l’Allegato III e gli artt. 5, 6 e 50 AI Act, separabilità dalle altre funzioni. Approfondire le qualificazioni normative che lo richiedono. Il lavoro da completare è questa analisi documentata delle funzioni esistenti.</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
         <x:v>Catalogo di Vera
@@ -815,7 +840,7 @@
         <x:v>Artt. 2 par. 12, 5, 6, 50 e All. III AI Act</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="92" customHeight="1">
+    <x:row r="18" ht="225" customHeight="1">
       <x:c r="A18" s="14" t="str">
         <x:v>G1.13 — Versionamento, registro delle modifiche e indicazione della licenza</x:v>
       </x:c>
@@ -823,14 +848,17 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C18" s="14" t="str">
-        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.</x:v>
+        <x:v>Vera è open source: il codice è consultabile nel repository, insieme alla licenza e alla cronologia delle modifiche. Il manifest dichiara la versione.
+Abbiamo considerato la possibilità di offrire a pagamento il servizio server di attestazione tecnica dei report e non la escludiamo. Allo stato riteniamo però che, per gran parte degli utilizzatori, un servizio aggiuntivo di questo tipo possa risultare largamente ridondante: Vera è open source e il suo funzionamento, compresi elaborazione locale e minimizzazione dei dati, è documentato e verificabile. Questa è la nostra valutazione della sua utilità commerciale. L’eventuale attestazione avrebbe per oggetto l’esistenza e l’integrità del report.</x:v>
       </x:c>
       <x:c r="D18" s="14" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="E18" s="22" t="str">
-        <x:v>Manifest Vera 0.1.338, repository e AGPL-3.0-only
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/.codex-plugin/plugin.json</x:v>
+        <x:v>Manifest corrente di Vera, repository e AGPL-3.0-only
+https://github.com/fabioannovazzi/app_files/blob/main/plugins/vera/.codex-plugin/plugin.json
+Licenza, servizi e modello economico: valutazione commerciale di Mparanza aggiornata al 07/10/2026.
+https://mparanza.com/static/shared/vera-compliance/index.html#attestazione-servizio</x:v>
       </x:c>
       <x:c r="F18" s="14" t="inlineStr">
         <x:is>
@@ -869,126 +897,125 @@
         <x:v>Art. 50, par. 2 AI Act; art. 111, par. 4 (Reg. UE 2026/1744)</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="92" customHeight="1">
+    <x:row r="20" ht="220" customHeight="1">
       <x:c r="A20" s="14" t="str">
+        <x:v>G1.15 — Descrizione unica e coerente delle funzioni e dei limiti d’uso in documentazione, termini d’uso e comunicazione pubblica</x:v>
+      </x:c>
+      <x:c r="B20" s="18" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12.</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E20" s="22" t="str">
+        <x:v>Funzioni e limiti d’uso: https://mparanza.com/terms#vera-functions-and-limits
+Ricevute: https://mparanza.com/zero-retention#run-receipts
+Catalogo: https://mparanza.com/static/shared/vera/index.html?lang=it
+Integrazioni: https://mparanza.com/static/shared/vera-integrazioni/index.html</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>Coerenza della descrizione delle funzioni e dei limiti d’uso fra documentazione, termini e comunicazione pubblica.</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>Art. 3, punto 12 AI Act; documento di orientamento della Commissione, parr. 10-14 (riferimenti dello schema di osservazioni).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="92" customHeight="1">
+      <x:c r="A21" s="13" t="str">
         <x:v>D2.1 — Bozza di registro dei trattamenti alimentata dai report di elaborazione</x:v>
       </x:c>
-      <x:c r="B20" s="18" t="str">
+      <x:c r="B21" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C21" s="13" t="str">
         <x:v>I report di Vera possono fornire informazioni sulle lavorazioni svolte e sui dati utilizzati.</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="D21" s="13" t="str">
         <x:v>Implementare la generazione di una bozza del registro dei trattamenti, integrando i report di Vera con le informazioni fornite dallo studio.</x:v>
       </x:c>
-      <x:c r="E20" s="22" t="str">
+      <x:c r="E21" s="21" t="str">
         <x:v>Report di esecuzione e dati già disponibili
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/references/model-data-report-contract.md</x:v>
       </x:c>
-      <x:c r="F20" s="14" t="inlineStr">
+      <x:c r="F21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supportare l'adempimento dell'art. 30</x:t>
         </x:is>
       </x:c>
-      <x:c r="G20" s="14" t="inlineStr">
+      <x:c r="G21" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 30 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="21" ht="92" customHeight="1">
-      <x:c r="A21" s="13" t="str">
+    <x:row r="22" ht="92" customHeight="1">
+      <x:c r="A22" s="14" t="str">
         <x:v>D2.2 — Scheda di screening preliminare per la DPIA</x:v>
       </x:c>
-      <x:c r="B21" s="17" t="str">
+      <x:c r="B22" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C22" s="14" t="str">
         <x:v>Vera dispone di percorsi di raccolta delle informazioni e analisi con fonti; la scheda dedicata di screening DPIA resta da implementare.</x:v>
       </x:c>
-      <x:c r="D21" s="13" t="str">
+      <x:c r="D22" s="14" t="str">
         <x:v>Implementare un percorso guidato che raccolga i fatti sul trattamento, li valuti rispetto ai criteri pertinenti e produca una scheda di screening DPIA motivata, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E21" s="21" t="str">
+      <x:c r="E22" s="22" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F21" s="13" t="inlineStr">
+      <x:c r="F22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Orientare la valutazione sulla necessità della DPIA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G21" s="13" t="inlineStr">
+      <x:c r="G22" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 35 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="22" ht="92" customHeight="1">
-      <x:c r="A22" s="14" t="str">
+    <x:row r="23" ht="92" customHeight="1">
+      <x:c r="A23" s="13" t="str">
         <x:v>D2.3 — Bozza di informativa ai clienti con clausola sull'uso dell'IA</x:v>
       </x:c>
-      <x:c r="B22" s="18" t="str">
+      <x:c r="B23" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C22" s="14" t="str">
+      <x:c r="C23" s="13" t="str">
         <x:v>New Client raccoglie informazioni privacy/IA e prepara un piano documentale; non produce la bozza dell’informativa richiesta.</x:v>
       </x:c>
-      <x:c r="D22" s="14" t="str">
+      <x:c r="D23" s="13" t="str">
         <x:v>Implementare la generazione di una bozza di informativa ai clienti con clausola sull’uso dell’IA, sulla base delle informazioni dello studio e delle fonti pertinenti, da sottoporre alla revisione del professionista.</x:v>
       </x:c>
-      <x:c r="E22" s="22" t="str">
+      <x:c r="E23" s="21" t="str">
         <x:v>Applicabilità privacy/IA e piano documentale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/new-client/skills/new-client/SKILL.md</x:v>
       </x:c>
-      <x:c r="F22" s="14" t="inlineStr">
+      <x:c r="F23" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Informativa privacy e informativa IA</x:t>
         </x:is>
       </x:c>
-      <x:c r="G22" s="14" t="inlineStr">
+      <x:c r="G23" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 13-14 GDPR; art. 13, co. 2, L. 132/2025; Informativa CNDCEC 156/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="92" customHeight="1">
-      <x:c r="A23" s="13" t="str">
-        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
-      </x:c>
-      <x:c r="B23" s="17" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C23" s="13" t="str">
-        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D23" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E23" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F23" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G23" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="92" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+        <x:v>D2.4 — Checklist di verifica del DPA del provider e bozza di eventuali nomine a responsabile</x:v>
       </x:c>
       <x:c r="B24" s="18" t="str">
         <x:v>Fuori perimetro</x:v>
       </x:c>
       <x:c r="C24" s="14" t="str">
-        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+        <x:v>La verifica del DPA del provider e le eventuali nomine a responsabile riguardano i rapporti contrattuali con il provider, esclusi dal perimetro concordato per Vera.</x:v>
       </x:c>
       <x:c r="D24" s="14" t="str">
         <x:v>—</x:v>
@@ -998,373 +1025,433 @@
       </x:c>
       <x:c r="F24" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+          <x:t xml:space="preserve">Verificare i contenuti minimi dell'atto di nomina (art. 28, par. 3, lett. a-h)</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Capo V GDPR</x:t>
+          <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="25" ht="92" customHeight="1">
       <x:c r="A25" s="13" t="str">
+        <x:v>D2.5 — Scheda precompilata per la valutazione dei trasferimenti extra-UE per ciascun provider</x:v>
+      </x:c>
+      <x:c r="B25" s="17" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="str">
+        <x:v>La valutazione dei trasferimenti extra-UE riguarda il provider scelto e le sue condizioni contrattuali e di trattamento dei dati, escluse dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D25" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E25" s="21" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F25" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Supportare la valutazione dei trasferimenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="13" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Capo V GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="92" customHeight="1">
+      <x:c r="A26" s="14" t="str">
         <x:v>D2.6 — Modello di policy IA di studio e registro degli usi dell'IA</x:v>
       </x:c>
-      <x:c r="B25" s="17" t="str">
+      <x:c r="B26" s="18" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="C26" s="14" t="str">
         <x:v>I report delle lavorazioni possono alimentare il registro degli usi di Vera. Le scelte per la policy e gli eventuali usi di altri strumenti IA sono forniti dallo studio.</x:v>
       </x:c>
-      <x:c r="D25" s="13" t="str">
+      <x:c r="D26" s="14" t="str">
         <x:v>Implementare il riepilogo degli usi di Vera dai report e la generazione di una bozza di policy IA basata sulle scelte dello studio, integrando gli altri usi dichiarati dallo studio.</x:v>
       </x:c>
-      <x:c r="E25" s="21" t="str">
+      <x:c r="E26" s="22" t="str">
         <x:v>Supporto generale a quesiti e bozze professionali
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F25" s="13" t="inlineStr">
+      <x:c r="F26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Governo dell'uso dell'IA nello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="13" t="inlineStr">
+      <x:c r="G26" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">AI Act (art. 4 nel testo modificato dal Reg. UE 2026/1744); L. 132/2025; Informativa CNDCEC 156/2025</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="26" ht="92" customHeight="1">
-      <x:c r="A26" s="14" t="str">
+    <x:row r="27" ht="92" customHeight="1">
+      <x:c r="A27" s="13" t="str">
         <x:v>D2.7 — Traccia per il registro della formazione/alfabetizzazione IA dei collaboratori</x:v>
       </x:c>
-      <x:c r="B26" s="18" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C26" s="14" t="str">
+      <x:c r="B27" s="17" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="str">
         <x:v>Vera offre corsi guidati sulle proprie funzioni e conserva localmente una traccia delle lezioni, delle esercitazioni e dei progressi dell’utente, utilizzabile per documentare la formazione svolta con Vera.</x:v>
       </x:c>
-      <x:c r="D26" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E26" s="22" t="str">
+      <x:c r="D27" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
         <x:v>Percorso didattico e registrazione locale dei progressi: sorgente locale esaminato
 /Users/fabio/Documents/GitHub/app_files/plugins/vera/skills/learn-with-vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F26" s="14" t="inlineStr">
+      <x:c r="F27" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dimostrare le attività di alfabetizzazione</x:t>
         </x:is>
       </x:c>
-      <x:c r="G26" s="14" t="inlineStr">
+      <x:c r="G27" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 AI Act (testo modificato)</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="92" customHeight="1">
-      <x:c r="A27" s="13" t="str">
-        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
-      </x:c>
-      <x:c r="B27" s="17" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C27" s="13" t="str">
-        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D27" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E27" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F27" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G27" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="28" ht="92" customHeight="1">
       <x:c r="A28" s="14" t="str">
+        <x:v>D2.8 — Bozza di procedura per la gestione di violazioni dei dati (rilevazione, notifica entro 72 ore, comunicazione agli interessati)</x:v>
+      </x:c>
+      <x:c r="B28" s="18" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>La procedura generale dello studio per la gestione delle violazioni dei dati è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E28" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preparare la risposta a incidenti</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Artt. 33-34 GDPR</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="135" customHeight="1">
+      <x:c r="A29" s="13" t="str">
         <x:v>D2.9 — Testo standard di disclosure sull'uso dell'IA da apporre agli elaborati</x:v>
       </x:c>
-      <x:c r="B28" s="18" t="str">
+      <x:c r="B29" s="17" t="str">
         <x:v>Da implementare</x:v>
       </x:c>
-      <x:c r="C28" s="14" t="str">
+      <x:c r="C29" s="13" t="str">
         <x:v>L’inserimento di un testo standard sull’uso dell’IA negli elaborati resta da implementare.</x:v>
       </x:c>
-      <x:c r="D28" s="14" t="str">
-        <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel.</x:v>
-      </x:c>
-      <x:c r="E28" s="22" t="str">
+      <x:c r="D29" s="13" t="str">
+        <x:v>Definire il testo e gli elaborati interessati e inserirlo nei modelli di output: nota nel documento Word/PDF o nel foglio principale dell’Excel. Da decidere: inserimento automatico per impostazione predefinita e possibilità per lo studio di modificarne il testo.</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
         <x:v>Provenienza dei workflow e redazione professionale
 https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/skills/vera/SKILL.md</x:v>
       </x:c>
-      <x:c r="F28" s="14" t="inlineStr">
+      <x:c r="F29" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Supporto alla trasparenza verso clienti e terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G28" s="14" t="inlineStr">
+      <x:c r="G29" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13, co. 2, L. 132/2025</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="92" customHeight="1">
-      <x:c r="A29" s="13" t="str">
-        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
-      </x:c>
-      <x:c r="B29" s="24" t="str">
-        <x:v>Fuori perimetro</x:v>
-      </x:c>
-      <x:c r="C29" s="13" t="str">
-        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
-      </x:c>
-      <x:c r="D29" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E29" s="21" t="str">
-        <x:v>Perimetro concordato nella revisione.</x:v>
-      </x:c>
-      <x:c r="F29" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G29" s="13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="30" ht="92" customHeight="1">
       <x:c r="A30" s="14" t="str">
+        <x:v>D2.10 — Checklist per autorizzati (art. 29) e amministratore di sistema</x:v>
+      </x:c>
+      <x:c r="B30" s="25" t="str">
+        <x:v>Fuori perimetro</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>La checklist per le persone autorizzate e l’amministratore di sistema riguarda l’organizzazione dello studio ed è esclusa dal perimetro concordato per Vera.</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E30" s="22" t="str">
+        <x:v>Perimetro concordato nella revisione.</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Istruzioni e designazioni all'interno dello studio</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="14" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Art. 29 GDPR; art. 2-quaterdecies Codice privacy; Provv. Garante 27/11/2008</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="92" customHeight="1">
+      <x:c r="A31" s="13" t="str">
         <x:v>N3.1 — Dichiarazione che Vera non rende "conforme" lo studio, che resta titolare e deployer</x:v>
       </x:c>
-      <x:c r="B30" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C30" s="14" t="str">
+      <x:c r="B31" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera facilita il lavoro dello studio senza certificarne la conformità e senza sostituirne il ruolo di titolare e di utilizzatore professionale dell’IA.</x:v>
       </x:c>
-      <x:c r="D30" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E30" s="22" t="str">
+      <x:c r="D31" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E31" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.1
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-1</x:v>
       </x:c>
-      <x:c r="F30" s="14" t="inlineStr">
+      <x:c r="F31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare affidamento improprio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G30" s="14" t="inlineStr">
+      <x:c r="G31" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 4 n. 7, 24 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="31" ht="92" customHeight="1">
-      <x:c r="A31" s="13" t="str">
+    <x:row r="32" ht="92" customHeight="1">
+      <x:c r="A32" s="14" t="str">
         <x:v>N3.2 — Dichiarazione che Vera non sostituisce la sottoscrizione del DPA con il provider né ne garantisce il contenuto</x:v>
       </x:c>
-      <x:c r="B31" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="B32" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
         <x:v>La documentazione d’uso precisa che Vera non sostituisce il DPA con il fornitore della piattaforma AI, quando necessario, e non ne verifica né garantisce il contenuto.</x:v>
       </x:c>
-      <x:c r="D31" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E31" s="21" t="str">
+      <x:c r="D32" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E32" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.2
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-2</x:v>
       </x:c>
-      <x:c r="F31" s="13" t="inlineStr">
+      <x:c r="F32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire la responsabilità dello studio</x:t>
         </x:is>
       </x:c>
-      <x:c r="G31" s="13" t="inlineStr">
+      <x:c r="G32" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="32" ht="92" customHeight="1">
-      <x:c r="A32" s="14" t="str">
+    <x:row r="33" ht="92" customHeight="1">
+      <x:c r="A33" s="13" t="str">
         <x:v>N3.3 — Dichiarazione che la minimizzazione/pseudonimizzazione non equivale ad anonimizzazione irreversibile, salvo diversa evidenza tecnica</x:v>
       </x:c>
-      <x:c r="B32" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C32" s="14" t="str">
+      <x:c r="B33" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str">
         <x:v>La documentazione d’uso distingue minimizzazione e pseudonimizzazione dall’anonimizzazione e chiarisce che il collegamento opzionale a un motore esterno non attribuisce automaticamente al risultato la qualità di anonimo.</x:v>
       </x:c>
-      <x:c r="D32" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E32" s="22" t="str">
+      <x:c r="D33" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E33" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.3
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-3</x:v>
       </x:c>
-      <x:c r="F32" s="14" t="inlineStr">
+      <x:c r="F33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare l'affidamento sull'"anonimo"</x:t>
         </x:is>
       </x:c>
-      <x:c r="G32" s="14" t="inlineStr">
+      <x:c r="G33" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 4 n. 5 GDPR; considerando 26</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="33" ht="92" customHeight="1">
-      <x:c r="A33" s="13" t="str">
+    <x:row r="34" ht="92" customHeight="1">
+      <x:c r="A34" s="14" t="str">
         <x:v>N3.4 — Dichiarazione che l'uso con account consumer o piani senza DPA non è coperto</x:v>
       </x:c>
-      <x:c r="B33" s="24" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="B34" s="25" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
         <x:v>La documentazione d’uso delimita il perimetro professionale descritto, escludendo account consumer e piani privi del DPA necessario. Il controllo dell’account non è una funzione di Vera.</x:v>
       </x:c>
-      <x:c r="D33" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E33" s="21" t="str">
+      <x:c r="D34" s="14" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E34" s="22" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.4
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-4</x:v>
       </x:c>
-      <x:c r="F33" s="13" t="inlineStr">
+      <x:c r="F34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Delimitare il perimetro d'uso</x:t>
         </x:is>
       </x:c>
-      <x:c r="G33" s="13" t="inlineStr">
+      <x:c r="G34" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 28 GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="34" ht="92" customHeight="1">
-      <x:c r="A34" s="14" t="str">
+    <x:row r="35" ht="92" customHeight="1">
+      <x:c r="A35" s="13" t="str">
         <x:v>N3.5 — Dichiarazione che Vera non controlla né garantisce regimi, residenza dei dati e trasferimenti dei provider</x:v>
       </x:c>
-      <x:c r="B34" s="25" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C34" s="14" t="str">
+      <x:c r="B35" s="24" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="str">
         <x:v>La documentazione d’uso chiarisce che Vera non controlla né garantisce conservazione, uso per addestramento, localizzazione e trasferimenti dei dati presso il fornitore della piattaforma AI.</x:v>
       </x:c>
-      <x:c r="D34" s="14" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E34" s="22" t="str">
+      <x:c r="D35" s="13" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E35" s="21" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.5
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-5</x:v>
       </x:c>
-      <x:c r="F34" s="14" t="inlineStr">
+      <x:c r="F35" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Chiarire i limiti rispetto ai terzi</x:t>
         </x:is>
       </x:c>
-      <x:c r="G34" s="14" t="inlineStr">
+      <x:c r="G35" s="13" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Artt. 28, 44 ss. GDPR</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="35" ht="92" customHeight="1">
-      <x:c r="A35" s="15" t="str">
+    <x:row r="36" ht="92" customHeight="1">
+      <x:c r="A36" s="11" t="str">
         <x:v>N3.6 — Dichiarazione che gli output non sono pareri professionali e restano sotto la responsabilità del professionista</x:v>
       </x:c>
-      <x:c r="B35" s="26" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C35" s="15" t="str">
+      <x:c r="B36" s="31" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C36" s="11" t="str">
         <x:v>La documentazione d’uso precisa che gli output, comprese le bozze di pareri, richiedono verifica e approvazione del professionista, che mantiene il giudizio e la responsabilità dell’elaborato finale.</x:v>
       </x:c>
-      <x:c r="D35" s="15" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E35" s="23" t="str">
+      <x:c r="D36" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E36" s="32" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.6
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-6</x:v>
       </x:c>
-      <x:c r="F35" s="15" t="inlineStr">
+      <x:c r="F36" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Prevalenza del giudizio umano</x:t>
         </x:is>
       </x:c>
-      <x:c r="G35" s="15" t="inlineStr">
+      <x:c r="G36" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Art. 13 L. 132/2025; art. 21 Codice deontologico CNDCEC</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="36" ht="92" customHeight="1">
-      <x:c r="A36" s="3" t="str">
+    <x:row r="37" ht="92" customHeight="1">
+      <x:c r="A37" s="3" t="str">
         <x:v>N3.7 — Avviso sull'aggiornamento normativo: data di verifica dei riferimenti e invito alla verifica sulle fonti ufficiali</x:v>
       </x:c>
-      <x:c r="B36" s="28" t="str">
-        <x:v>Presente</x:v>
-      </x:c>
-      <x:c r="C36" s="3" t="str">
+      <x:c r="B37" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C37" s="3" t="str">
         <x:v>L’avviso indica il 4 ottobre 2026 come data di consultazione delle fonti delle sette dichiarazioni e invita a verificare il testo vigente sulle fonti ufficiali prima dell’utilizzo professionale.</x:v>
       </x:c>
-      <x:c r="D36" s="3" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E36" s="29" t="str">
+      <x:c r="D37" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E37" s="29" t="str">
         <x:v>Condizioni e limiti d’uso di Vera — N3.7
 https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-7</x:v>
       </x:c>
-      <x:c r="F36" s="3" t="inlineStr">
+      <x:c r="F37" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Evitare obsolescenza non dichiarata</x:t>
         </x:is>
       </x:c>
-      <x:c r="G36" s="3" t="inlineStr">
+      <x:c r="G37" s="3" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="37" ht="150" customHeight="1">
-      <x:c r="A37" s="3" t="str">
+    <x:row r="38" ht="150" customHeight="1">
+      <x:c r="A38" s="3" t="str">
         <x:v>N3.8 — Dichiarazione del piano utilizzato all'avvio ed elenco dei presidi che Vera non copre, riportati anche nella documentazione d'uso</x:v>
       </x:c>
-      <x:c r="B37" s="28" t="str">
+      <x:c r="B38" s="28" t="str">
         <x:v>Non previsto</x:v>
       </x:c>
-      <x:c r="C37" s="3" t="str">
+      <x:c r="C38" s="3" t="str">
         <x:v>Vera non richiede una dichiarazione del piano utilizzato all’avvio. Le condizioni d’uso pubblicate elencano già i limiti relativi a contratti, account, trattamento dei dati sulla piattaforma e revisione professionale. La scelta del piano resta esterna a Vera, come indicato in G1.6.</x:v>
       </x:c>
-      <x:c r="D37" s="3" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E37" s="29" t="str">
+      <x:c r="D38" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E38" s="29" t="str">
         <x:v>Condizioni e limiti già pubblicati
 https://mparanza.com/static/shared/vera-compliance/index.html#condizioni-uso
 Piattaforma e piano utilizzato
 https://mparanza.com/static/shared/vera-compliance/index.html#g1-6</x:v>
       </x:c>
-      <x:c r="F37" s="3" t="str">
+      <x:c r="F38" s="3" t="str">
         <x:v>Informare lo studio di ciò che resta a suo carico</x:v>
       </x:c>
-      <x:c r="G37" s="3" t="str">
+      <x:c r="G38" s="3" t="str">
         <x:v>Artt. 4 n. 7, 24, 28 GDPR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="405" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>N3.9 — Dichiarazione sul servizio delle ricevute tecniche</x:v>
+      </x:c>
+      <x:c r="B39" s="28" t="str">
+        <x:v>Presente</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>Vera calcola sul computer l’hash SHA-256 del report: una stringa di 64 caratteri. È un’impronta per confrontare documenti, non una copia cifrata del report: non esiste un’operazione di decifratura che ne restituisca il contenuto.
+Il comando che genera il report con ricevuta invia automaticamente solo quell’impronta, la versione dello schema, un ID casuale della ricevuta e la versione di Vera. Non invia report, documenti del cliente, nomi dei file, prompt o risposte del modello.
+Mparanza firma la prova con la data del server. Chi possiede il report può ricalcolarne l’hash sul proprio computer e confrontarlo con la prova firmata: la verifica non richiede l’invio del report a Mparanza. Il servizio opera in Finlandia e conserva la prova senza scadenza automatica.
+Mparanza non riceve nomi o identificativi dei clienti né la corrispondenza fra hash e persone. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo. Non prevediamo un interruttore per disattivare l’invio della ricevuta: non aggiungerebbe protezione ai contenuti del fascicolo, che non vengono trasmessi. L’invio automatico crea la prova tecnica. I log di connessione sono distinti e descritti separatamente.</x:v>
+      </x:c>
+      <x:c r="D39" s="3" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E39" s="29" t="str">
+        <x:v>Dichiarazione N3.9
+https://mparanza.com/static/shared/vera-compliance/index.html#condizione-n3-9
+Descrizione del servizio e dei log
+https://mparanza.com/zero-retention#run-receipts
+Log distinti dalle ricevute: IP, URL ed esito HTTP. L’URL può includere ID della ricevuta e hash; non contiene report o documenti. L’IP serve a limitare richieste eccessive e non è nel database delle ricevute.
+Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.
+Mparanza LLC opera come titolare autonomo per i log tecnici del proprio servizio, con finalità di sicurezza e prevenzione degli abusi. La base giuridica individuata è il legittimo interesse (art. 6, par. 1, lett. f, GDPR), nei limiti di necessità e proporzionalità. Referente e rappresentante di Mparanza LLC: Fabio Annovazzi, Anières (Svizzera).
+Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>Descrivere agli studi il funzionamento e i dati del servizio di ricevuta tecnica.</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
+        <x:v>Artt. 13, 28 GDPR (riferimenti indicati nello schema di osservazioni).</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1375,7 +1462,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd233c18d27424f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re99f4807f93640c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: describe anonymous Vera incident recovery in compliance materials
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Ra36cc176fb9649f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7d53ae8446d843a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 07/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 13/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -617,22 +617,21 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>Il report resta locale. Vera ne calcola l’hash SHA-256: un’impronta di 64 caratteri, non una copia cifrata. Invia automaticamente hash, versione dello schema, ID casuale della ricevuta e versione di Vera. Non invia report, documenti, nomi dei file, prompt o output del modello. La verifica confronta l’hash ricalcolato localmente con la prova firmata (N3.9).
-Mparanza non riceve nomi dei clienti né una corrispondenza fra hash e persone. L’ID identifica la ricevuta. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo (considerando 26): l’invio crea la prova tecnica senza comunicare i contenuti.
-Il servizio opera e conserva le ricevute in Finlandia (UE); Mparanza LLC è costituita in Delaware.
-L’IP non serve alla ricevuta e non è salvato nel suo database. L’endpoint lo usa per limitare richieste eccessive; i log degli accessi lo registrano separatamente.
-Nginx conserva 14 archivi giornalieri più il corrente. Per il log Uvicorn non risulta un termine massimo; lo script lo sovrascrive al riavvio.
-La prova firmata è conservata senza scadenza automatica. Le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
+        <x:v>I contenuti delle lavorazioni sono esclusi dagli invii a Mparanza.
+Ricevuta tecnica: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report e documenti restano locali. Funzionamento, Finlandia, log e conservazione sono descritti in N3.9.
+Diagnosi e risoluzione degli errori tecnici: invio automatico delle informazioni tecniche del guasto, escludendo documenti, prompt, elaborati, credenziali e informazioni personali. Collegamento anonimo con ID casuale, senza account nominativo. Il monitoraggio periodico con AI esamina gli errori aperti. La stessa installazione recupera il rimedio e comunica l’esito. Il problema si chiude quando l’operazione interrotta riesce.
+Le segnalazioni dei guasti sono distinte dalle richieste di nuove funzioni.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>build_receipt_request(): quattro campi ammessi
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py
-Configurazione e log del server verificati il 07/10/2026.
-Conservazione della prova firmata: modules/run_receipts/store.py, schema e metodi stamp()/get(), verificati il 07/10/2026.
-Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.</x:v>
+        <x:v>Ricevute: quattro campi ammessi; descrizione e conservazione in N3.9. Log server verificati il 07/10/2026.
+Diagnosi e risoluzione degli errori tecnici:
+https://mparanza.com/static/shared/vera-compliance/index.html#diagnosi-errori
+Documentazione del servizio e dei dati trasmessi:
+https://github.com/fabioannovazzi/app_files/blob/3fbd29e58ad50c7e6db571ba45c6e604fea7eed2/plugins/vera/privacy/services/operational-incidents.json
+Il servizio seleziona le informazioni tecniche; non inoltra i log grezzi delle lavorazioni.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -1462,7 +1461,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re99f4807f93640c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17ed0d72994cc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: explain Vera incident diagnosis in compliance materials (#812)
* docs: describe anonymous Vera incident recovery in compliance materials

* style: separate incident service explanation paragraphs

---------

Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Ra36cc176fb9649f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7d53ae8446d843a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 07/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 13/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -617,22 +617,21 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>Il report resta locale. Vera ne calcola l’hash SHA-256: un’impronta di 64 caratteri, non una copia cifrata. Invia automaticamente hash, versione dello schema, ID casuale della ricevuta e versione di Vera. Non invia report, documenti, nomi dei file, prompt o output del modello. La verifica confronta l’hash ricalcolato localmente con la prova firmata (N3.9).
-Mparanza non riceve nomi dei clienti né una corrispondenza fra hash e persone. L’ID identifica la ricevuta. Su questi presupposti considera le impronte anonime rispetto alle persone del fascicolo (considerando 26): l’invio crea la prova tecnica senza comunicare i contenuti.
-Il servizio opera e conserva le ricevute in Finlandia (UE); Mparanza LLC è costituita in Delaware.
-L’IP non serve alla ricevuta e non è salvato nel suo database. L’endpoint lo usa per limitare richieste eccessive; i log degli accessi lo registrano separatamente.
-Nginx conserva 14 archivi giornalieri più il corrente. Per il log Uvicorn non risulta un termine massimo; lo script lo sovrascrive al riavvio.
-La prova firmata è conservata senza scadenza automatica. Le istruzioni per il feedback escludono i materiali dei clienti.</x:v>
+        <x:v>I contenuti delle lavorazioni sono esclusi dagli invii a Mparanza.
+Ricevuta tecnica: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report e documenti restano locali. Funzionamento, Finlandia, log e conservazione sono descritti in N3.9.
+Diagnosi e risoluzione degli errori tecnici: invio automatico delle informazioni tecniche del guasto, escludendo documenti, prompt, elaborati, credenziali e informazioni personali. Collegamento anonimo con ID casuale, senza account nominativo. Il monitoraggio periodico con AI esamina gli errori aperti. La stessa installazione recupera il rimedio e comunica l’esito. Il problema si chiude quando l’operazione interrotta riesce.
+Le segnalazioni dei guasti sono distinte dalle richieste di nuove funzioni.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>build_receipt_request(): quattro campi ammessi
-https://github.com/fabioannovazzi/app_files/blob/0736b552e3cdc117d0b61324e72310cdfaac8d5f/plugins/vera/scripts/notarized_run_receipt.py
-Configurazione e log del server verificati il 07/10/2026.
-Conservazione della prova firmata: modules/run_receipts/store.py, schema e metodi stamp()/get(), verificati il 07/10/2026.
-Nginx conserva 14 archivi giornalieri più il file corrente. Per il log dell’applicazione Uvicorn non è stata individuata una durata massima prefissata; lo script operativo lo sovrascrive a ogni riavvio.</x:v>
+        <x:v>Ricevute: quattro campi ammessi; descrizione e conservazione in N3.9. Log server verificati il 07/10/2026.
+Diagnosi e risoluzione degli errori tecnici:
+https://mparanza.com/static/shared/vera-compliance/index.html#diagnosi-errori
+Documentazione del servizio e dei dati trasmessi:
+https://github.com/fabioannovazzi/app_files/blob/3fbd29e58ad50c7e6db571ba45c6e604fea7eed2/plugins/vera/privacy/services/operational-incidents.json
+Il servizio seleziona le informazioni tecniche; non inoltra i log grezzi delle lavorazioni.</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -1462,7 +1461,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re99f4807f93640c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17ed0d72994cc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: describe Vera usage and satisfaction monitoring
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7d53ae8446d843a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdd9f2ce214cd4e44"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 13/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 17/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -617,21 +617,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>I contenuti delle lavorazioni sono esclusi dagli invii a Mparanza.
-Ricevuta tecnica: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report e documenti restano locali. Funzionamento, Finlandia, log e conservazione sono descritti in N3.9.
-Diagnosi e risoluzione degli errori tecnici: invio automatico delle informazioni tecniche del guasto, escludendo documenti, prompt, elaborati, credenziali e informazioni personali. Collegamento anonimo con ID casuale, senza account nominativo. Il monitoraggio periodico con AI esamina gli errori aperti. La stessa installazione recupera il rimedio e comunica l’esito. Il problema si chiude quando l’operazione interrotta riesce.
-Le segnalazioni dei guasti sono distinte dalle richieste di nuove funzioni.</x:v>
+        <x:v>Gli eventi tecnici escludono documenti, prompt, elaborati e contenuti delle lavorazioni.
+Ricevuta: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report locale; Finlandia, log e conservazione in N3.9.
+Guasti: diagnosi automatica con informazioni tecniche selezionate, ID casuale senza account nominativo e monitoraggio AI. La stessa installazione recupera il rimedio e comunica se l’operazione interrotta riesce. Le richieste di nuove funzioni sono separate.
+Uso e soddisfazione: invio automatico di processo, applicazione, versione, date ed esito, con ID casuale dell’installazione. Esito non osservato: sconosciuto. Stelle da 1 a 5 e commento facoltativi per migliorare Vera; nessuna risposta: nessuna valutazione. Studio Archive e test non aumentano l’uso ordinario. Possibile collegamento alla ricevuta senza inviare il report. Servizio in Finlandia; eventi e feedback conservati fino a cancellazione amministrativa, senza scadenza automatica.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>Ricevute: quattro campi ammessi; descrizione e conservazione in N3.9. Log server verificati il 07/10/2026.
-Diagnosi e risoluzione degli errori tecnici:
+        <x:v>Ricevute, log e conservazione: N3.9. Log verificati il 07/10/2026.
+Diagnosi e risoluzione dei guasti:
 https://mparanza.com/static/shared/vera-compliance/index.html#diagnosi-errori
-Documentazione del servizio e dei dati trasmessi:
-https://github.com/fabioannovazzi/app_files/blob/3fbd29e58ad50c7e6db571ba45c6e604fea7eed2/plugins/vera/privacy/services/operational-incidents.json
-Il servizio seleziona le informazioni tecniche; non inoltra i log grezzi delle lavorazioni.</x:v>
+Uso, esiti, soddisfazione e conservazione:
+https://mparanza.com/static/shared/vera-compliance/index.html#monitoraggio-utilizzo
+Campi trasmessi e funzionamento:
+https://github.com/fabioannovazzi/app_files/blob/1e8a87934/plugins/vera/privacy/services/workflow-usage.json</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -904,7 +905,7 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12.</x:v>
+        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12. È descritto anche il monitoraggio anonimo dell’uso, degli esiti e della soddisfazione.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
         <x:v>—</x:v>
@@ -1461,7 +1462,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17ed0d72994cc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22f188ddb15f41d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: describe Vera usage and satisfaction monitoring (#855)
* docs: describe Vera usage and satisfaction monitoring

* fix: include monitoring disclosure in every data page language

* chore: align Clara privacy review with usage disclosures

---------

Co-authored-by: fabio annovazzi <3429553+fabioannovazzi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
+++ b/static/shared/vera-compliance/downloads/riscontro-vera.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="R7d53ae8446d843a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscontro" sheetId="1" r:id="Rdd9f2ce214cd4e44"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 13/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
+        <x:v>Schema di riferimento: versione 0.2 del 03/10/2026 e osservazioni G1.15 e N3.9 del 04/10/2026. Versione di lavoro per il confronto, aggiornata al 17/10/2026; evidenze e attività proposte indicate per ciascuna voce. Il connettore di anonimizzazione è opzionale.</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
       <x:c r="C3" s="5"/>
@@ -617,21 +617,22 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>I contenuti delle lavorazioni sono esclusi dagli invii a Mparanza.
-Ricevuta tecnica: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report e documenti restano locali. Funzionamento, Finlandia, log e conservazione sono descritti in N3.9.
-Diagnosi e risoluzione degli errori tecnici: invio automatico delle informazioni tecniche del guasto, escludendo documenti, prompt, elaborati, credenziali e informazioni personali. Collegamento anonimo con ID casuale, senza account nominativo. Il monitoraggio periodico con AI esamina gli errori aperti. La stessa installazione recupera il rimedio e comunica l’esito. Il problema si chiude quando l’operazione interrotta riesce.
-Le segnalazioni dei guasti sono distinte dalle richieste di nuove funzioni.</x:v>
+        <x:v>Gli eventi tecnici escludono documenti, prompt, elaborati e contenuti delle lavorazioni.
+Ricevuta: invio automatico di hash SHA-256, versione dello schema, ID casuale e versione di Vera. Report locale; Finlandia, log e conservazione in N3.9.
+Guasti: diagnosi automatica con informazioni tecniche selezionate, ID casuale senza account nominativo e monitoraggio AI. La stessa installazione recupera il rimedio e comunica se l’operazione interrotta riesce. Le richieste di nuove funzioni sono separate.
+Uso e soddisfazione: invio automatico di processo, applicazione, versione, date ed esito, con ID casuale dell’installazione. Esito non osservato: sconosciuto. Stelle da 1 a 5 e commento facoltativi per migliorare Vera; nessuna risposta: nessuna valutazione. Studio Archive e test non aumentano l’uso ordinario. Possibile collegamento alla ricevuta senza inviare il report. Servizio in Finlandia; eventi e feedback conservati fino a cancellazione amministrativa, senza scadenza automatica.</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Da attuare: limite di conservazione di 14 giorni, con cancellazione automatica dei log tecnici. Le ricevute firmate restano escluse da questa cancellazione.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>Ricevute: quattro campi ammessi; descrizione e conservazione in N3.9. Log server verificati il 07/10/2026.
-Diagnosi e risoluzione degli errori tecnici:
+        <x:v>Ricevute, log e conservazione: N3.9. Log verificati il 07/10/2026.
+Diagnosi e risoluzione dei guasti:
 https://mparanza.com/static/shared/vera-compliance/index.html#diagnosi-errori
-Documentazione del servizio e dei dati trasmessi:
-https://github.com/fabioannovazzi/app_files/blob/3fbd29e58ad50c7e6db571ba45c6e604fea7eed2/plugins/vera/privacy/services/operational-incidents.json
-Il servizio seleziona le informazioni tecniche; non inoltra i log grezzi delle lavorazioni.</x:v>
+Uso, esiti, soddisfazione e conservazione:
+https://mparanza.com/static/shared/vera-compliance/index.html#monitoraggio-utilizzo
+Campi trasmessi e funzionamento:
+https://github.com/fabioannovazzi/app_files/blob/1e8a87934/plugins/vera/privacy/services/workflow-usage.json</x:v>
       </x:c>
       <x:c r="F10" s="14" t="inlineStr">
         <x:is>
@@ -904,7 +905,7 @@
         <x:v>Presente</x:v>
       </x:c>
       <x:c r="C20" s="14" t="str">
-        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12.</x:v>
+        <x:v>Allineate le descrizioni delle funzioni e dei limiti d’uso nei termini e nelle pagine pubbliche: funzioni e limiti dei processi, piattaforme, cinque motori opzionali senza raccomandazione di Mparanza, report locale e ricevuta tecnica, localizzazione e conservazione, condizioni dell’assistenza. I testi rimandano al catalogo e alle descrizioni dei singoli processi. L’analisi normativa delle funzioni resta separata in G1.12. È descritto anche il monitoraggio anonimo dell’uso, degli esiti e della soddisfazione.</x:v>
       </x:c>
       <x:c r="D20" s="14" t="str">
         <x:v>—</x:v>
@@ -1461,7 +1462,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c17ed0d72994cc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22f188ddb15f41d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>